<commit_message>
Use measured 30-day ad spend instead of extrapolating
The 30-day product ad spend was estimated as 7-day actuals x 30/7, which
triples the figure for campaigns that started mid-window. 卓上冷感クーラー
(started 7/13) was reported as 84,521 JPY in the red when it is actually
472,286 JPY in the black; 5WAY, ポンチョ and ムダ毛 were wrong the same way.

Pull the 30-day campaign totals in a single query instead, and add section
5c so this is not repeated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-26.xlsx
+++ b/data/reports/report-2026-07-26.xlsx
@@ -138,8 +138,8 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績）</t>
+          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・30日広告費を実測に訂正）</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
         <v>545552</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>460941</v>
+        <v>463968</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -664,7 +664,7 @@
         <v>457498</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>450934</v>
+        <v>447908</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -696,7 +696,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>35.1%</t>
+          <t>34.8%</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -722,7 +722,7 @@
         <v>407165</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>406076</v>
+        <v>403050</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -890,22 +890,22 @@
         <v>11203643</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>13828236</v>
+        <v>13919026</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>13528022</v>
+        <v>13437232</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.351</v>
+        <v>0.348</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>1345741</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>12182281</v>
+        <v>12091491</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.316</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="18">
@@ -942,40 +942,47 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>・売上=gross_sales−discounts（返品A案）。当月返品累計 7/25時点 187,481円（返品率0.58%）。7/25 新規返品ゼロ</t>
+          <t>・★訂正: 30日の商品別広告費を「7日実績×30/7」で外挿していたのを実測値に修正。7/13開始の卓上冷感クーラー等、期間途中で開始した商品の利益が大幅に過小評価されていた</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>・★7/26判定: 湯上がりガーゼワンピースは余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
+          <t>・売上=gross_sales−discounts（返品A案）。当月返品累計 7/25時点 187,481円（返品率0.58%）。7/25 新規返品ゼロ</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>・★曜日指数を30日実測で更新: 日116・水106・土103・月97・金97・木94・火87</t>
+          <t>・★7/26判定: 湯上がりガーゼワンピースは余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>・30日利益率 35.08% で目標35%を達成。7日は31.72%</t>
+          <t>・★曜日指数を30日実測で更新: 日116・水106・土103・月97・金97・木94・火87</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>・増分MERは7/22以降に予算を3,000円/日以上動かした商品がないため今回は全商品「判定保留」。7/28の増額判定時に再測定する</t>
+          <t>・30日利益率 35.08% で目標35%を達成。7日は31.72%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>・増分MERは7/22以降に予算を3,000円/日以上動かした商品がないため今回は全商品「判定保留」。7/28の増額判定時に再測定する</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>・予算はMetaライブ実測（4WAY 95,000円・ディスペンサー 6,000円）</t>
         </is>
@@ -1168,7 +1175,7 @@
         <v>377498</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>1925169</v>
+        <v>2697046</v>
       </c>
       <c r="O2" s="9" t="n">
         <v>3.94</v>
@@ -1237,7 +1244,7 @@
         <v>227928</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>2135671</v>
+        <v>2127799</v>
       </c>
       <c r="O3" s="14" t="n">
         <v>3.43</v>
@@ -1306,7 +1313,7 @@
         <v>240571</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>3506104</v>
+        <v>3921630</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>2.78</v>
@@ -1375,7 +1382,7 @@
         <v>147288</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>2151144</v>
+        <v>2240654</v>
       </c>
       <c r="O5" s="14" t="n">
         <v>2.39</v>
@@ -1445,8 +1452,8 @@
       <c r="M6" s="5" t="n">
         <v>127525</v>
       </c>
-      <c r="N6" s="17" t="n">
-        <v>-84521</v>
+      <c r="N6" s="5" t="n">
+        <v>472286</v>
       </c>
       <c r="O6" s="9" t="n">
         <v>3.95</v>
@@ -1517,7 +1524,7 @@
         <v>81658</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>703148</v>
+        <v>916606</v>
       </c>
       <c r="O7" s="14" t="n">
         <v>2.7</v>
@@ -1586,7 +1593,7 @@
         <v>86873</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>622760</v>
+        <v>760675</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>2.85</v>
@@ -1656,8 +1663,8 @@
       <c r="M9" s="12" t="n">
         <v>54272</v>
       </c>
-      <c r="N9" s="18" t="n">
-        <v>-80211</v>
+      <c r="N9" s="12" t="n">
+        <v>170979</v>
       </c>
       <c r="O9" s="14" t="n">
         <v>5.15</v>
@@ -1721,14 +1728,14 @@
       <c r="K10" s="17" t="n">
         <v>-5878</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="L10" s="18" t="n">
         <v>-0.328</v>
       </c>
       <c r="M10" s="17" t="n">
         <v>-4867</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>136243</v>
+        <v>218247</v>
       </c>
       <c r="O10" s="9" t="n">
         <v>2.99</v>
@@ -1789,17 +1796,17 @@
       <c r="J11" s="12" t="n">
         <v>19900</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>-3946</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="L11" s="18" t="n">
         <v>-0.198</v>
       </c>
       <c r="M11" s="12" t="n">
         <v>15962</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>563979</v>
+        <v>567535</v>
       </c>
       <c r="O11" s="14" t="n">
         <v>1.73</v>
@@ -1869,8 +1876,8 @@
       <c r="M12" s="5" t="n">
         <v>10688</v>
       </c>
-      <c r="N12" s="17" t="n">
-        <v>-124720</v>
+      <c r="N12" s="5" t="n">
+        <v>55759</v>
       </c>
       <c r="O12" s="9" t="n">
         <v>2.5</v>
@@ -1941,7 +1948,7 @@
         <v>42617</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>363339</v>
+        <v>394568</v>
       </c>
       <c r="O13" s="14" t="n">
         <v>1.91</v>
@@ -2011,8 +2018,8 @@
       <c r="M14" s="5" t="n">
         <v>58558</v>
       </c>
-      <c r="N14" s="17" t="n">
-        <v>-67623</v>
+      <c r="N14" s="5" t="n">
+        <v>133083</v>
       </c>
       <c r="O14" s="9" t="n">
         <v>2.29</v>
@@ -2083,7 +2090,7 @@
         <v>27295</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>319053</v>
+        <v>320815</v>
       </c>
       <c r="O15" s="14" t="n">
         <v>1.97</v>
@@ -2154,7 +2161,7 @@
         <v>-5049</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>252045</v>
+        <v>207251</v>
       </c>
       <c r="O16" s="9" t="n">
         <v>2.08</v>
@@ -2225,7 +2232,7 @@
         <v>21990</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>292200</v>
+        <v>270885</v>
       </c>
       <c r="O17" s="14" t="n">
         <v>1.67</v>
@@ -2269,7 +2276,7 @@
       <c r="E18" s="17" t="n">
         <v>-22107</v>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F18" s="18" t="n">
         <v>-0.2195</v>
       </c>
       <c r="G18" s="8" t="n">
@@ -2289,14 +2296,14 @@
       <c r="K18" s="17" t="n">
         <v>-2096</v>
       </c>
-      <c r="L18" s="19" t="n">
+      <c r="L18" s="18" t="n">
         <v>-0.15</v>
       </c>
       <c r="M18" s="17" t="n">
         <v>-4689</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>276683</v>
+        <v>104670</v>
       </c>
       <c r="O18" s="9" t="n">
         <v>1.16</v>
@@ -2357,15 +2364,15 @@
       <c r="J19" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="18" t="n">
+      <c r="K19" s="19" t="n">
         <v>-5379</v>
       </c>
       <c r="L19" s="11" t="inlineStr"/>
-      <c r="M19" s="18" t="n">
+      <c r="M19" s="19" t="n">
         <v>-13821</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>245757</v>
+        <v>106500</v>
       </c>
       <c r="O19" s="14" t="n">
         <v>1.66</v>
@@ -2436,7 +2443,7 @@
         <v>115</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>195020</v>
+        <v>96139</v>
       </c>
       <c r="O20" s="9" t="n">
         <v>1.52</v>

</xml_diff>

<commit_message>
Rebuild the 07-26 report on measured data only
Make "measured data only" the skill's top-level rule and remove the
remaining approximations from today's report:

- 30-day cost now uses actual per-variant quantities rather than the
  7-day mix applied to 30-day totals
- The 7/18 cumulative row used a 7-day average in place of 7/18's own
  cost (439,069 vs the actual 374,937), which overstated 8-day COGS
- 30-day ad spend stays on the measured campaign totals from yesterday

Also flag campaigns whose start date falls inside the 30-day window so
their 30-day profit is not compared against full-window products.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-26.xlsx
+++ b/data/reports/report-2026-07-26.xlsx
@@ -522,7 +522,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・30日広告費を実測に訂正）</t>
+          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・全期間Meta/Shopify実測）</t>
         </is>
       </c>
     </row>
@@ -887,13 +887,13 @@
         <v>38559901</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>11203643</v>
+        <v>11203519</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>13919026</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>13437232</v>
+        <v>13437356</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>0.348</v>
@@ -902,7 +902,7 @@
         <v>1345741</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>12091491</v>
+        <v>12091615</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0.314</v>
@@ -918,45 +918,45 @@
         <v>11417483</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>3513080</v>
+        <v>3448948</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>4321489</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>3582914</v>
+        <v>3647046</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>0.314</v>
+        <v>0.319</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>398470</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>3184444</v>
+        <v>3248576</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.279</v>
+        <v>0.285</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>・★訂正: 30日の商品別広告費を「7日実績×30/7」で外挿していたのを実測値に修正。7/13開始の卓上冷感クーラー等、期間途中で開始した商品の利益が大幅に過小評価されていた</t>
+          <t>・売上=gross_sales−discounts（返品A案）。当月返品累計 7/25時点 187,481円（返品率0.58%）。7/25 新規返品ゼロ</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>・売上=gross_sales−discounts（返品A案）。当月返品累計 7/25時点 187,481円（返品率0.58%）。7/25 新規返品ゼロ</t>
+          <t>・★全期間の広告費・原価をMeta/Shopifyの実測に統一（推計・外挿を全廃）。30日広告費は実測13,919,026円、30日原価はバリエーション別実数量、7/18累積は7/18の実原価374,937円を使用</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>・★7/26判定: 湯上がりガーゼワンピースは余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
+          <t>・★7/26判定: 湯上がりガーゼワンピースは7日余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
         </is>
       </c>
     </row>
@@ -970,21 +970,21 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>・30日利益率 35.08% で目標35%を達成。7日は31.72%</t>
+          <t>・30日利益率 34.80%（目標35%まであと0.2pt）。7日は31.72%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>・増分MERは7/22以降に予算を3,000円/日以上動かした商品がないため今回は全商品「判定保留」。7/28の増額判定時に再測定する</t>
+          <t>・増分MER: 7/22以降に予算を3,000円/日以上動かした商品がないため今回は全商品「判定保留」。7/28の増額判定時に再測定</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>・予算はMetaライブ実測（4WAY 95,000円・ディスペンサー 6,000円）</t>
+          <t>・30日窓の途中で開始した商品は稼働日数が短い: 卓上冷感クーラー7/13開始(13日)・5WAY腰掛けファン7/19開始(7日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10開始(16日)</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
         <v>147288</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>2240654</v>
+        <v>2239920</v>
       </c>
       <c r="O5" s="14" t="n">
         <v>2.39</v>
@@ -2303,7 +2303,7 @@
         <v>-4689</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>104670</v>
+        <v>105528</v>
       </c>
       <c r="O18" s="9" t="n">
         <v>1.16</v>

</xml_diff>

<commit_message>
Group the product sheet by period and add the target MER column
Reading the sheet meant jumping between interleaved 前日 and 3日 columns,
and 3日利益率 was blank for most rows because it was limited to products
selling 20+ units a day.

- Order the columns 7日 → 3日 → 前日, each carrying the same five figures
- Show 3日利益率 for every product; the volume caveat stays in the notes
- Surface 目標MER per product and shade MER green/red against it

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-26.xlsx
+++ b/data/reports/report-2026-07-26.xlsx
@@ -59,7 +59,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EFD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -125,6 +130,7 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -137,6 +143,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -505,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -522,7 +529,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・全期間Meta/Shopify実測）</t>
+          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・7日/3日/前日を並列表示）</t>
         </is>
       </c>
     </row>
@@ -949,42 +956,56 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>・★全期間の広告費・原価をMeta/Shopifyの実測に統一（推計・外挿を全廃）。30日広告費は実測13,919,026円、30日原価はバリエーション別実数量、7/18累積は7/18の実原価374,937円を使用</t>
+          <t>・★列を「7日 → 3日 → 前日」の順に並べ替え、3日も売上/原価/広告費/利益/利益率の5項目に拡張（前日も同じ5項目に統一）</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>・★7/26判定: 湯上がりガーゼワンピースは7日余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
+          <t>・★目標MER列を追加。目標MER = 1 ÷ (1 − その商品の原価率 − 0.35)。商品ごとに2.17〜5.49と差が大きいため全店値2.91は使わない。MER列は目標超え=緑・未達=赤</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>・★曜日指数を30日実測で更新: 日116・水106・土103・月97・金97・木94・火87</t>
+          <t>・★3日利益率は全商品に表示（従来は日販20個以上に限定）。ただし日販10個未満の商品は日次のブレが13〜64ptあり、3日平均でも実力を測れない点は変わらない</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>・30日利益率 34.80%（目標35%まであと0.2pt）。7日は31.72%</t>
+          <t>・★7/26判定: 湯上がりガーゼワンピースは7日余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>・増分MER: 7/22以降に予算を3,000円/日以上動かした商品がないため今回は全商品「判定保留」。7/28の増額判定時に再測定</t>
+          <t>・★増額候補（自分の目標MER超え×消化率95%以上）: 害虫ブロッカー(2.78&gt;2.31・102%)・ナノガラス脱毛パッド(2.39&gt;2.17・100%)・完全遮光(2.70&gt;2.56・95%)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>・30日窓の途中で開始した商品は稼働日数が短い: 卓上冷感クーラー7/13開始(13日)・5WAY腰掛けファン7/19開始(7日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10開始(16日)</t>
+          <t>・全期間の広告費・原価はMeta/Shopifyの実測。推計・外挿は不使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>・30日窓の途中開始: 卓上冷感クーラー7/13(13日)・5WAY腰掛けファン7/19(7日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10(16日)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>・増分MER: 7/22以降に予算を3,000円/日以上動かした商品がないため全商品「判定保留」</t>
         </is>
       </c>
     </row>
@@ -999,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:AA28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1010,19 +1031,25 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="52" customWidth="1" min="21" max="21"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="7" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="52" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1068,65 +1095,95 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
+          <t>3日売上</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>3日原価</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>3日広告費</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>3日利益</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
           <t>3日利益率</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>前日売上</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>前日原価</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>前日広告費</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>前日利益</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>前日利益率</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>3日利益</t>
-        </is>
-      </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>30日利益</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>MER(7日)</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>分岐</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>目標MER</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>余裕</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>増分MER</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>現日予算(円)</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>推奨アクション</t>
         </is>
@@ -1159,112 +1216,148 @@
       <c r="H2" s="6" t="n">
         <v>0.2538</v>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="5" t="n">
+        <v>976080</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>339080</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>259502</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>377498</v>
+      </c>
+      <c r="M2" s="6" t="n">
         <v>0.3867</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="N2" s="5" t="n">
         <v>348600</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="O2" s="5" t="n">
+        <v>121100</v>
+      </c>
+      <c r="P2" s="5" t="n">
+        <v>87318</v>
+      </c>
+      <c r="Q2" s="5" t="n">
         <v>140182</v>
       </c>
-      <c r="L2" s="6" t="n">
-        <v>0.402</v>
-      </c>
-      <c r="M2" s="5" t="n">
-        <v>377498</v>
-      </c>
-      <c r="N2" s="5" t="n">
+      <c r="R2" s="6" t="n">
+        <v>0.4021</v>
+      </c>
+      <c r="S2" s="5" t="n">
         <v>2697046</v>
       </c>
-      <c r="O2" s="9" t="n">
+      <c r="T2" s="9" t="n">
         <v>3.94</v>
       </c>
-      <c r="P2" s="9" t="n">
+      <c r="U2" s="10" t="n">
         <v>1.53</v>
       </c>
-      <c r="Q2" s="9" t="n">
+      <c r="V2" s="10" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="W2" s="10" t="n">
         <v>2.41</v>
       </c>
-      <c r="R2" s="4" t="inlineStr"/>
-      <c r="S2" s="5" t="n">
+      <c r="X2" s="4" t="inlineStr"/>
+      <c r="Y2" s="5" t="n">
         <v>95000</v>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>✅95k初日(7/28判定)</t>
         </is>
       </c>
-      <c r="U2" s="10" t="inlineStr">
+      <c r="AA2" s="11" t="inlineStr">
         <is>
           <t>①7/25に95kへ増額。消化率90%で余裕あり→7/28に増分MER≥2.91なら110k ②原価率34.7%。月1,344個の最大SKU＝CJ数量交渉の最有力 ③+500円値上げは13.3%減まで許容</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>形状記憶日傘</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="13" t="n">
         <v>1439220</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="13" t="n">
         <v>378301</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="13" t="n">
         <v>419790</v>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="E3" s="13" t="n">
         <v>641129</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="14" t="n">
         <v>0.4455</v>
       </c>
-      <c r="G3" s="13" t="n">
+      <c r="G3" s="14" t="n">
         <v>0.2629</v>
       </c>
-      <c r="H3" s="13" t="n">
+      <c r="H3" s="14" t="n">
         <v>0.2917</v>
       </c>
       <c r="I3" s="13" t="n">
+        <v>537840</v>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>141372</v>
+      </c>
+      <c r="K3" s="13" t="n">
+        <v>168540</v>
+      </c>
+      <c r="L3" s="13" t="n">
+        <v>227928</v>
+      </c>
+      <c r="M3" s="14" t="n">
         <v>0.4238</v>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="N3" s="13" t="n">
         <v>219120</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="O3" s="13" t="n">
+        <v>57596</v>
+      </c>
+      <c r="P3" s="13" t="n">
+        <v>54689</v>
+      </c>
+      <c r="Q3" s="13" t="n">
         <v>106835</v>
       </c>
-      <c r="L3" s="13" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>227928</v>
-      </c>
-      <c r="N3" s="12" t="n">
+      <c r="R3" s="14" t="n">
+        <v>0.4876</v>
+      </c>
+      <c r="S3" s="13" t="n">
         <v>2127799</v>
       </c>
-      <c r="O3" s="14" t="n">
+      <c r="T3" s="9" t="n">
         <v>3.43</v>
       </c>
-      <c r="P3" s="14" t="n">
+      <c r="U3" s="15" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q3" s="14" t="n">
+      <c r="V3" s="15" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="W3" s="15" t="n">
         <v>2.07</v>
       </c>
-      <c r="R3" s="11" t="inlineStr"/>
-      <c r="S3" s="12" t="n">
+      <c r="X3" s="12" t="inlineStr"/>
+      <c r="Y3" s="13" t="n">
         <v>60000</v>
       </c>
-      <c r="T3" s="11" t="inlineStr">
+      <c r="Z3" s="12" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="U3" s="15" t="inlineStr">
+      <c r="AA3" s="16" t="inlineStr">
         <is>
           <t>①MER3.43・余裕+2.07に改善、消化率93%。据置 ②原価率26.3%・広告費率29.2%とも健全 ③お盆明け(8/15)から段階減額の計画を</t>
         </is>
@@ -1297,112 +1390,148 @@
       <c r="H4" s="6" t="n">
         <v>0.3593</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="5" t="n">
+        <v>589040</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>128316</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>220153</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>240571</v>
+      </c>
+      <c r="M4" s="6" t="n">
         <v>0.4084</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="N4" s="5" t="n">
         <v>199000</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="O4" s="5" t="n">
+        <v>43350</v>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>77160</v>
+      </c>
+      <c r="Q4" s="5" t="n">
         <v>78490</v>
       </c>
-      <c r="L4" s="6" t="n">
-        <v>0.394</v>
-      </c>
-      <c r="M4" s="5" t="n">
-        <v>240571</v>
-      </c>
-      <c r="N4" s="5" t="n">
+      <c r="R4" s="6" t="n">
+        <v>0.3944</v>
+      </c>
+      <c r="S4" s="5" t="n">
         <v>3921630</v>
       </c>
-      <c r="O4" s="9" t="n">
+      <c r="T4" s="9" t="n">
         <v>2.78</v>
       </c>
-      <c r="P4" s="9" t="n">
+      <c r="U4" s="10" t="n">
         <v>1.28</v>
       </c>
-      <c r="Q4" s="9" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="R4" s="4" t="inlineStr"/>
-      <c r="S4" s="5" t="n">
+      <c r="V4" s="10" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="W4" s="10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="X4" s="4" t="inlineStr"/>
+      <c r="Y4" s="5" t="n">
         <v>73000</v>
       </c>
-      <c r="T4" s="4" t="inlineStr">
+      <c r="Z4" s="4" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="U4" s="10" t="inlineStr">
+      <c r="AA4" s="11" t="inlineStr">
         <is>
           <t>①消化率102%で天井張り付き。ただしMER2.78&lt;目標2.91＝増額は率を薄める。据置 ②原価率21.7%は最良 ③30日利益の最大の稼ぎ頭。触らないのが最善</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>ナノガラス脱毛パッド</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="13" t="n">
         <v>899480</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>169773</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="13" t="n">
         <v>376745</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="13" t="n">
         <v>352962</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="14" t="n">
         <v>0.3924</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="14" t="n">
         <v>0.1887</v>
       </c>
       <c r="H5" s="8" t="n">
         <v>0.4188</v>
       </c>
       <c r="I5" s="13" t="n">
+        <v>398000</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>75105</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>175607</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <v>147288</v>
+      </c>
+      <c r="M5" s="14" t="n">
         <v>0.3701</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="N5" s="13" t="n">
         <v>163180</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="O5" s="13" t="n">
+        <v>30782</v>
+      </c>
+      <c r="P5" s="13" t="n">
+        <v>61455</v>
+      </c>
+      <c r="Q5" s="13" t="n">
         <v>70943</v>
       </c>
-      <c r="L5" s="13" t="n">
-        <v>0.435</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>147288</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>2239920</v>
-      </c>
-      <c r="O5" s="14" t="n">
+      <c r="R5" s="14" t="n">
+        <v>0.4348</v>
+      </c>
+      <c r="S5" s="13" t="n">
+        <v>2241388</v>
+      </c>
+      <c r="T5" s="9" t="n">
         <v>2.39</v>
       </c>
-      <c r="P5" s="14" t="n">
+      <c r="U5" s="15" t="n">
         <v>1.23</v>
       </c>
-      <c r="Q5" s="14" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="R5" s="11" t="inlineStr"/>
-      <c r="S5" s="12" t="n">
+      <c r="V5" s="15" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="W5" s="15" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="X5" s="12" t="inlineStr"/>
+      <c r="Y5" s="13" t="n">
         <v>60000</v>
       </c>
-      <c r="T5" s="11" t="inlineStr">
+      <c r="Z5" s="12" t="inlineStr">
         <is>
           <t>✅BC検証中</t>
         </is>
       </c>
-      <c r="U5" s="15" t="inlineStr">
+      <c r="AA5" s="16" t="inlineStr">
         <is>
           <t>①消化率100%天井だが余裕+1.15・MER2.39と目標未達。BC検証の結果待ち ②原価率18.9%は全商品最良、広告費率41.9%が重し ③通年需要＝秋以降の主力候補</t>
         </is>
@@ -1435,116 +1564,148 @@
       <c r="H6" s="6" t="n">
         <v>0.2533</v>
       </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I6" s="5" t="n">
+        <v>334880</v>
       </c>
       <c r="J6" s="5" t="n">
+        <v>111776</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>95579</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>127525</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>0.3808</v>
+      </c>
+      <c r="N6" s="5" t="n">
         <v>53820</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="O6" s="5" t="n">
+        <v>17964</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>35525</v>
+      </c>
+      <c r="Q6" s="5" t="n">
         <v>331</v>
       </c>
-      <c r="L6" s="16" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>127525</v>
-      </c>
-      <c r="N6" s="5" t="n">
+      <c r="R6" s="17" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="S6" s="5" t="n">
         <v>472286</v>
       </c>
-      <c r="O6" s="9" t="n">
+      <c r="T6" s="9" t="n">
         <v>3.95</v>
       </c>
-      <c r="P6" s="9" t="n">
+      <c r="U6" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="Q6" s="9" t="n">
+      <c r="V6" s="10" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="W6" s="10" t="n">
         <v>2.45</v>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="5" t="n">
+      <c r="X6" s="4" t="inlineStr"/>
+      <c r="Y6" s="5" t="n">
         <v>38000</v>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="Z6" s="4" t="inlineStr">
         <is>
           <t>✅消化率88%回復(7/27判定)</t>
         </is>
       </c>
-      <c r="U6" s="10" t="inlineStr">
+      <c r="AA6" s="11" t="inlineStr">
         <is>
           <t>①消化率79%→88%に回復。7/27に増分MER判定 ②原価率33.4%。+500円値上げは11.2%減まで許容 ③MER3.95・余裕+2.45と好調</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>完全遮光・形状記憶・晴雨兼用・UV日傘</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="13" t="n">
         <v>702180</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="13" t="n">
         <v>181951</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="13" t="n">
         <v>260052</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <v>260177</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <v>0.3705</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="14" t="n">
         <v>0.2591</v>
       </c>
-      <c r="H7" s="13" t="n">
+      <c r="H7" s="14" t="n">
         <v>0.3703</v>
       </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="n">
+      <c r="I7" s="13" t="n">
+        <v>268920</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>69377</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>117885</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>81658</v>
+      </c>
+      <c r="M7" s="14" t="n">
+        <v>0.3037</v>
+      </c>
+      <c r="N7" s="13" t="n">
         <v>49800</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="O7" s="13" t="n">
+        <v>11781</v>
+      </c>
+      <c r="P7" s="13" t="n">
+        <v>37609</v>
+      </c>
+      <c r="Q7" s="13" t="n">
         <v>410</v>
       </c>
-      <c r="L7" s="16" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="M7" s="12" t="n">
-        <v>81658</v>
-      </c>
-      <c r="N7" s="12" t="n">
+      <c r="R7" s="17" t="n">
+        <v>0.008200000000000001</v>
+      </c>
+      <c r="S7" s="13" t="n">
         <v>916606</v>
       </c>
-      <c r="O7" s="14" t="n">
+      <c r="T7" s="9" t="n">
         <v>2.7</v>
       </c>
-      <c r="P7" s="14" t="n">
+      <c r="U7" s="15" t="n">
         <v>1.35</v>
       </c>
-      <c r="Q7" s="14" t="n">
+      <c r="V7" s="15" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="W7" s="15" t="n">
         <v>1.35</v>
       </c>
-      <c r="R7" s="11" t="inlineStr"/>
-      <c r="S7" s="12" t="n">
+      <c r="X7" s="12" t="inlineStr"/>
+      <c r="Y7" s="13" t="n">
         <v>41000</v>
       </c>
-      <c r="T7" s="11" t="inlineStr">
+      <c r="Z7" s="12" t="inlineStr">
         <is>
           <t>👀余裕+1.35(7/28判定)</t>
         </is>
       </c>
-      <c r="U7" s="15" t="inlineStr">
+      <c r="AA7" s="16" t="inlineStr">
         <is>
           <t>①余裕+1.82→+1.35に低下、MER3.17→2.70。7/28判定で増分MER&lt;2.91なら据置確定 ②日傘2本合算MER3.20 ③8/15から減額</t>
         </is>
@@ -1568,7 +1729,7 @@
       <c r="E8" s="5" t="n">
         <v>178079</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <v>0.2887</v>
       </c>
       <c r="G8" s="8" t="n">
@@ -1577,114 +1738,148 @@
       <c r="H8" s="6" t="n">
         <v>0.351</v>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I8" s="5" t="n">
+        <v>290540</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>104682</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>98985</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>86873</v>
+      </c>
+      <c r="M8" s="17" t="n">
         <v>0.299</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="N8" s="5" t="n">
         <v>83580</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="O8" s="5" t="n">
+        <v>30114</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>34385</v>
+      </c>
+      <c r="Q8" s="5" t="n">
         <v>19081</v>
       </c>
-      <c r="L8" s="16" t="n">
-        <v>0.228</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>86873</v>
-      </c>
-      <c r="N8" s="5" t="n">
+      <c r="R8" s="17" t="n">
+        <v>0.2283</v>
+      </c>
+      <c r="S8" s="5" t="n">
         <v>760675</v>
       </c>
-      <c r="O8" s="9" t="n">
+      <c r="T8" s="18" t="n">
         <v>2.85</v>
       </c>
-      <c r="P8" s="9" t="n">
+      <c r="U8" s="10" t="n">
         <v>1.56</v>
       </c>
-      <c r="Q8" s="9" t="n">
+      <c r="V8" s="10" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="W8" s="10" t="n">
         <v>1.29</v>
       </c>
-      <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="5" t="n">
+      <c r="X8" s="4" t="inlineStr"/>
+      <c r="Y8" s="5" t="n">
         <v>34000</v>
       </c>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="Z8" s="4" t="inlineStr">
         <is>
           <t>⚠️利益率28.9%(7/28判定)</t>
         </is>
       </c>
-      <c r="U8" s="10" t="inlineStr">
+      <c r="AA8" s="11" t="inlineStr">
         <is>
           <t>①利益率35.0%→28.9%に悪化、消化率98%天井。7/28判定 ②原価率36.0%。売価3,980円で+500円値上げは16.4%減まで許容＝値上げ余地最大 ③CR疲弊の可能性→素材があれば投入</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>5WAY腰掛けファン</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="13" t="n">
         <v>393420</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="13" t="n">
         <v>145992</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="13" t="n">
         <v>76449</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="13" t="n">
         <v>170979</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="14" t="n">
         <v>0.4346</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>0.3711</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="14" t="n">
         <v>0.1943</v>
       </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
+      <c r="I9" s="13" t="n">
+        <v>144420</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>53592</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>36556</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>54272</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>0.3758</v>
+      </c>
+      <c r="N9" s="13" t="n">
         <v>59760</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="O9" s="13" t="n">
+        <v>22176</v>
+      </c>
+      <c r="P9" s="13" t="n">
+        <v>12036</v>
+      </c>
+      <c r="Q9" s="13" t="n">
         <v>25548</v>
       </c>
-      <c r="L9" s="13" t="n">
-        <v>0.428</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>54272</v>
-      </c>
-      <c r="N9" s="12" t="n">
+      <c r="R9" s="14" t="n">
+        <v>0.4275</v>
+      </c>
+      <c r="S9" s="13" t="n">
         <v>170979</v>
       </c>
-      <c r="O9" s="14" t="n">
+      <c r="T9" s="9" t="n">
         <v>5.15</v>
       </c>
-      <c r="P9" s="14" t="n">
+      <c r="U9" s="15" t="n">
         <v>1.59</v>
       </c>
-      <c r="Q9" s="14" t="n">
+      <c r="V9" s="15" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="W9" s="15" t="n">
         <v>3.56</v>
       </c>
-      <c r="R9" s="11" t="inlineStr"/>
-      <c r="S9" s="12" t="n">
+      <c r="X9" s="12" t="inlineStr"/>
+      <c r="Y9" s="13" t="n">
         <v>13000</v>
       </c>
-      <c r="T9" s="11" t="inlineStr">
+      <c r="Z9" s="12" t="inlineStr">
         <is>
           <t>👀学習中(7/28判定)</t>
         </is>
       </c>
-      <c r="U9" s="15" t="inlineStr">
+      <c r="AA9" s="16" t="inlineStr">
         <is>
           <t>①MER5.15・余裕+3.56で全商品最高効率。消化率92% ②広告費率19.4%は最良＝伸びしろ最大。7/28判定で増額候補 ③原価率37.1%が唯一の弱点</t>
         </is>
@@ -1708,7 +1903,7 @@
       <c r="E10" s="5" t="n">
         <v>76293</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <v>0.2502</v>
       </c>
       <c r="G10" s="8" t="n">
@@ -1717,116 +1912,148 @@
       <c r="H10" s="6" t="n">
         <v>0.3343</v>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I10" s="5" t="n">
+        <v>71760</v>
       </c>
       <c r="J10" s="5" t="n">
+        <v>29820</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>46807</v>
+      </c>
+      <c r="L10" s="19" t="n">
+        <v>-4867</v>
+      </c>
+      <c r="M10" s="20" t="n">
+        <v>-0.0678</v>
+      </c>
+      <c r="N10" s="5" t="n">
         <v>17940</v>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="O10" s="5" t="n">
+        <v>7455</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>16363</v>
+      </c>
+      <c r="Q10" s="19" t="n">
         <v>-5878</v>
       </c>
-      <c r="L10" s="18" t="n">
-        <v>-0.328</v>
-      </c>
-      <c r="M10" s="17" t="n">
-        <v>-4867</v>
-      </c>
-      <c r="N10" s="5" t="n">
+      <c r="R10" s="20" t="n">
+        <v>-0.3276</v>
+      </c>
+      <c r="S10" s="5" t="n">
         <v>218247</v>
       </c>
-      <c r="O10" s="9" t="n">
+      <c r="T10" s="18" t="n">
         <v>2.99</v>
       </c>
-      <c r="P10" s="9" t="n">
+      <c r="U10" s="10" t="n">
         <v>1.71</v>
       </c>
-      <c r="Q10" s="9" t="n">
+      <c r="V10" s="10" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="W10" s="10" t="n">
         <v>1.28</v>
       </c>
-      <c r="R10" s="4" t="inlineStr"/>
-      <c r="S10" s="5" t="n">
+      <c r="X10" s="4" t="inlineStr"/>
+      <c r="Y10" s="5" t="n">
         <v>16000</v>
       </c>
-      <c r="T10" s="4" t="inlineStr">
+      <c r="Z10" s="4" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="U10" s="10" t="inlineStr">
+      <c r="AA10" s="11" t="inlineStr">
         <is>
           <t>①消化率101%天井・MER2.99。据置 ②原価率41.6%が主因で利益率25.0% ③5,980→6,980円の値上げは22.2%減まで許容＝値上げ最有力 ④CJ交渉で2,485→2,200円なら利益率+4.8pt</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>偏光・調光サングラス</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="13" t="n">
         <v>266660</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>59831</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>153852</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>52977</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="17" t="n">
         <v>0.1987</v>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="G11" s="14" t="n">
         <v>0.2244</v>
       </c>
       <c r="H11" s="8" t="n">
         <v>0.577</v>
       </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
+      <c r="I11" s="13" t="n">
+        <v>99500</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>22325</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>61213</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>15962</v>
+      </c>
+      <c r="M11" s="17" t="n">
+        <v>0.1604</v>
+      </c>
+      <c r="N11" s="13" t="n">
         <v>19900</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="O11" s="13" t="n">
+        <v>4465</v>
+      </c>
+      <c r="P11" s="13" t="n">
+        <v>19381</v>
+      </c>
+      <c r="Q11" s="21" t="n">
         <v>-3946</v>
       </c>
-      <c r="L11" s="18" t="n">
-        <v>-0.198</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>15962</v>
-      </c>
-      <c r="N11" s="12" t="n">
+      <c r="R11" s="20" t="n">
+        <v>-0.1983</v>
+      </c>
+      <c r="S11" s="13" t="n">
         <v>567535</v>
       </c>
-      <c r="O11" s="14" t="n">
+      <c r="T11" s="18" t="n">
         <v>1.73</v>
       </c>
-      <c r="P11" s="14" t="n">
+      <c r="U11" s="15" t="n">
         <v>1.29</v>
       </c>
-      <c r="Q11" s="14" t="n">
+      <c r="V11" s="15" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="W11" s="15" t="n">
         <v>0.44</v>
       </c>
-      <c r="R11" s="11" t="inlineStr"/>
-      <c r="S11" s="12" t="n">
+      <c r="X11" s="12" t="inlineStr"/>
+      <c r="Y11" s="13" t="n">
         <v>22000</v>
       </c>
-      <c r="T11" s="11" t="inlineStr">
+      <c r="Z11" s="12" t="inlineStr">
         <is>
           <t>⚠️余裕+0.80→+0.44に急落</t>
         </is>
       </c>
-      <c r="U11" s="15" t="inlineStr">
+      <c r="AA11" s="16" t="inlineStr">
         <is>
           <t>①7/25に購入2件と急落、7日余裕+0.80→+0.44。悪化トレンド ②原価率22.4%は健全、広告費率57.7%が主因＝広告の問題 ③7/29判定。CR差し替えが本命、素材がなければ複製リセット ④消化率90%</t>
         </is>
@@ -1850,7 +2077,7 @@
       <c r="E12" s="5" t="n">
         <v>30190</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="17" t="n">
         <v>0.1329</v>
       </c>
       <c r="G12" s="8" t="n">
@@ -1859,116 +2086,148 @@
       <c r="H12" s="6" t="n">
         <v>0.3993</v>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I12" s="5" t="n">
+        <v>83720</v>
       </c>
       <c r="J12" s="5" t="n">
+        <v>39172</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>33860</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>10688</v>
+      </c>
+      <c r="M12" s="17" t="n">
+        <v>0.1277</v>
+      </c>
+      <c r="N12" s="5" t="n">
         <v>35880</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="O12" s="5" t="n">
+        <v>16788</v>
+      </c>
+      <c r="P12" s="5" t="n">
+        <v>11441</v>
+      </c>
+      <c r="Q12" s="5" t="n">
         <v>7651</v>
       </c>
-      <c r="L12" s="16" t="n">
-        <v>0.213</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>10688</v>
-      </c>
-      <c r="N12" s="5" t="n">
+      <c r="R12" s="17" t="n">
+        <v>0.2132</v>
+      </c>
+      <c r="S12" s="5" t="n">
         <v>55759</v>
       </c>
-      <c r="O12" s="9" t="n">
+      <c r="T12" s="18" t="n">
         <v>2.5</v>
       </c>
-      <c r="P12" s="9" t="n">
+      <c r="U12" s="10" t="n">
         <v>1.88</v>
       </c>
-      <c r="Q12" s="9" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="R12" s="4" t="inlineStr"/>
-      <c r="S12" s="5" t="n">
+      <c r="V12" s="10" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="W12" s="10" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="X12" s="4" t="inlineStr"/>
+      <c r="Y12" s="5" t="n">
         <v>13000</v>
       </c>
-      <c r="T12" s="4" t="inlineStr">
+      <c r="Z12" s="4" t="inlineStr">
         <is>
           <t>✅黒字+30,190(7/27判定)</t>
         </is>
       </c>
-      <c r="U12" s="10" t="inlineStr">
+      <c r="AA12" s="11" t="inlineStr">
         <is>
           <t>①7日利益+30,190に改善、余裕+0.63。7/27判定 ②原価率46.8%が最大の問題＝広告では直らない ③5,980→6,980円値上げは23.9%減まで許容＝値上げ最優先候補 ④CJ原価2,798円は交渉余地あり</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>接触冷感UVアームカバー</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>226860</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>44688</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>118806</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>63366</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="17" t="n">
         <v>0.2793</v>
       </c>
-      <c r="G13" s="13" t="n">
+      <c r="G13" s="14" t="n">
         <v>0.197</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>0.5237000000000001</v>
       </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J13" s="12" t="n">
+      <c r="I13" s="13" t="n">
+        <v>115420</v>
+      </c>
+      <c r="J13" s="13" t="n">
+        <v>22736</v>
+      </c>
+      <c r="K13" s="13" t="n">
+        <v>50067</v>
+      </c>
+      <c r="L13" s="13" t="n">
+        <v>42617</v>
+      </c>
+      <c r="M13" s="14" t="n">
+        <v>0.3692</v>
+      </c>
+      <c r="N13" s="13" t="n">
         <v>47760</v>
       </c>
-      <c r="K13" s="12" t="n">
+      <c r="O13" s="13" t="n">
+        <v>9408</v>
+      </c>
+      <c r="P13" s="13" t="n">
+        <v>16054</v>
+      </c>
+      <c r="Q13" s="13" t="n">
         <v>22298</v>
       </c>
-      <c r="L13" s="13" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="M13" s="12" t="n">
-        <v>42617</v>
-      </c>
-      <c r="N13" s="12" t="n">
+      <c r="R13" s="14" t="n">
+        <v>0.4669</v>
+      </c>
+      <c r="S13" s="13" t="n">
         <v>394568</v>
       </c>
-      <c r="O13" s="14" t="n">
+      <c r="T13" s="18" t="n">
         <v>1.91</v>
       </c>
-      <c r="P13" s="14" t="n">
+      <c r="U13" s="15" t="n">
         <v>1.25</v>
       </c>
-      <c r="Q13" s="14" t="n">
+      <c r="V13" s="15" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="W13" s="15" t="n">
         <v>0.66</v>
       </c>
-      <c r="R13" s="11" t="inlineStr"/>
-      <c r="S13" s="12" t="n">
+      <c r="X13" s="12" t="inlineStr"/>
+      <c r="Y13" s="13" t="n">
         <v>17000</v>
       </c>
-      <c r="T13" s="11" t="inlineStr">
+      <c r="Z13" s="12" t="inlineStr">
         <is>
           <t>👀7/29判定</t>
         </is>
       </c>
-      <c r="U13" s="15" t="inlineStr">
+      <c r="AA13" s="16" t="inlineStr">
         <is>
           <t>①消化率98%天井だが余裕+0.66で増額ライン未達 ②原価率19.7%は極めて良い、広告費率52.4%が主因 ③売価3,980円でAOVが小さい→パーカー/UVハットとのセット販売が本命 ④7/29判定</t>
         </is>
@@ -2001,116 +2260,148 @@
       <c r="H14" s="8" t="n">
         <v>0.4373</v>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I14" s="5" t="n">
+        <v>127360</v>
       </c>
       <c r="J14" s="5" t="n">
+        <v>31584</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>37218</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>58558</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>0.4598</v>
+      </c>
+      <c r="N14" s="5" t="n">
         <v>27860</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="O14" s="5" t="n">
+        <v>6909</v>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>12949</v>
+      </c>
+      <c r="Q14" s="5" t="n">
         <v>8002</v>
       </c>
-      <c r="L14" s="16" t="n">
-        <v>0.287</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>58558</v>
-      </c>
-      <c r="N14" s="5" t="n">
+      <c r="R14" s="17" t="n">
+        <v>0.2872</v>
+      </c>
+      <c r="S14" s="5" t="n">
         <v>133083</v>
       </c>
-      <c r="O14" s="9" t="n">
+      <c r="T14" s="18" t="n">
         <v>2.29</v>
       </c>
-      <c r="P14" s="9" t="n">
+      <c r="U14" s="10" t="n">
         <v>1.33</v>
       </c>
-      <c r="Q14" s="9" t="n">
+      <c r="V14" s="10" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="W14" s="10" t="n">
         <v>0.96</v>
       </c>
-      <c r="R14" s="4" t="inlineStr"/>
-      <c r="S14" s="5" t="n">
+      <c r="X14" s="4" t="inlineStr"/>
+      <c r="Y14" s="5" t="n">
         <v>13000</v>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="Z14" s="4" t="inlineStr">
         <is>
           <t>✅余裕+0.96に改善</t>
         </is>
       </c>
-      <c r="U14" s="10" t="inlineStr">
+      <c r="AA14" s="11" t="inlineStr">
         <is>
           <t>①余裕+0.40→+0.96に改善、利益率31.5% ②消化率95%天井 ③原価率24.8%は良好 ④夏物で最も季節性が強い。8月中旬から縮小</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>健康サンダル</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="13" t="n">
         <v>179280</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="13" t="n">
         <v>39508</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <v>90907</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <v>48865</v>
       </c>
-      <c r="F15" s="16" t="n">
+      <c r="F15" s="17" t="n">
         <v>0.2726</v>
       </c>
-      <c r="G15" s="13" t="n">
+      <c r="G15" s="14" t="n">
         <v>0.2204</v>
       </c>
       <c r="H15" s="8" t="n">
         <v>0.5071</v>
       </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
+      <c r="I15" s="13" t="n">
+        <v>84660</v>
+      </c>
+      <c r="J15" s="13" t="n">
+        <v>17430</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>39935</v>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>27295</v>
+      </c>
+      <c r="M15" s="14" t="n">
+        <v>0.3224</v>
+      </c>
+      <c r="N15" s="13" t="n">
         <v>19920</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="O15" s="13" t="n">
+        <v>4648</v>
+      </c>
+      <c r="P15" s="13" t="n">
+        <v>13335</v>
+      </c>
+      <c r="Q15" s="13" t="n">
         <v>1937</v>
       </c>
-      <c r="L15" s="16" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>27295</v>
-      </c>
-      <c r="N15" s="12" t="n">
+      <c r="R15" s="17" t="n">
+        <v>0.09719999999999999</v>
+      </c>
+      <c r="S15" s="13" t="n">
         <v>320815</v>
       </c>
-      <c r="O15" s="14" t="n">
+      <c r="T15" s="18" t="n">
         <v>1.97</v>
       </c>
-      <c r="P15" s="14" t="n">
+      <c r="U15" s="15" t="n">
         <v>1.28</v>
       </c>
-      <c r="Q15" s="14" t="n">
+      <c r="V15" s="15" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="W15" s="15" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="R15" s="11" t="inlineStr"/>
-      <c r="S15" s="12" t="n">
+      <c r="X15" s="12" t="inlineStr"/>
+      <c r="Y15" s="13" t="n">
         <v>13000</v>
       </c>
-      <c r="T15" s="11" t="inlineStr">
+      <c r="Z15" s="12" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="U15" s="15" t="inlineStr">
+      <c r="AA15" s="16" t="inlineStr">
         <is>
           <t>①消化率102%天井、余裕+0.69 ②原価率22.0%は良好、広告費率50.7%が主因 ③18サイズ展開でサイズ選択UIの改善がCVR向上の本命 ④秋以降も需要継続する非季節商品</t>
         </is>
@@ -2134,7 +2425,7 @@
       <c r="E16" s="5" t="n">
         <v>28532</v>
       </c>
-      <c r="F16" s="16" t="n">
+      <c r="F16" s="17" t="n">
         <v>0.179</v>
       </c>
       <c r="G16" s="8" t="n">
@@ -2143,69 +2434,85 @@
       <c r="H16" s="8" t="n">
         <v>0.4819</v>
       </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I16" s="5" t="n">
+        <v>39840</v>
       </c>
       <c r="J16" s="5" t="n">
+        <v>13944</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>30945</v>
+      </c>
+      <c r="L16" s="19" t="n">
+        <v>-5049</v>
+      </c>
+      <c r="M16" s="20" t="n">
+        <v>-0.1267</v>
+      </c>
+      <c r="N16" s="5" t="n">
         <v>19920</v>
       </c>
-      <c r="K16" s="5" t="n">
+      <c r="O16" s="5" t="n">
+        <v>6972</v>
+      </c>
+      <c r="P16" s="5" t="n">
+        <v>10085</v>
+      </c>
+      <c r="Q16" s="5" t="n">
         <v>2863</v>
       </c>
-      <c r="L16" s="16" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>-5049</v>
-      </c>
-      <c r="N16" s="5" t="n">
+      <c r="R16" s="17" t="n">
+        <v>0.1437</v>
+      </c>
+      <c r="S16" s="5" t="n">
         <v>207251</v>
       </c>
-      <c r="O16" s="9" t="n">
+      <c r="T16" s="18" t="n">
         <v>2.08</v>
       </c>
-      <c r="P16" s="9" t="n">
+      <c r="U16" s="10" t="n">
         <v>1.51</v>
       </c>
-      <c r="Q16" s="9" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="5" t="n">
+      <c r="V16" s="10" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="W16" s="10" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="X16" s="4" t="inlineStr"/>
+      <c r="Y16" s="5" t="n">
         <v>11000</v>
       </c>
-      <c r="T16" s="4" t="inlineStr">
+      <c r="Z16" s="4" t="inlineStr">
         <is>
           <t>👀8/1判定</t>
         </is>
       </c>
-      <c r="U16" s="10" t="inlineStr">
+      <c r="AA16" s="11" t="inlineStr">
         <is>
           <t>①余裕+0.33→+0.56に改善、7日利益+28,532 ②日販4.4個でブレ±64pt＝利益率では判断不能、7日累計で見る ③8/1判定 ④原価率33.9%・広告費率48.2%の両方が重い</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>UV歯ブラシ除菌器</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="13" t="n">
         <v>134700</v>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="13" t="n">
         <v>48600</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="13" t="n">
         <v>80486</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="13" t="n">
         <v>5614</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F17" s="17" t="n">
         <v>0.0417</v>
       </c>
       <c r="G17" s="8" t="n">
@@ -2214,45 +2521,61 @@
       <c r="H17" s="8" t="n">
         <v>0.5975</v>
       </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
+      <c r="I17" s="13" t="n">
+        <v>80820</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>29160</v>
+      </c>
+      <c r="K17" s="13" t="n">
+        <v>29670</v>
+      </c>
+      <c r="L17" s="13" t="n">
+        <v>21990</v>
+      </c>
+      <c r="M17" s="17" t="n">
+        <v>0.2721</v>
+      </c>
+      <c r="N17" s="13" t="n">
         <v>35920</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="O17" s="13" t="n">
+        <v>12960</v>
+      </c>
+      <c r="P17" s="13" t="n">
+        <v>8224</v>
+      </c>
+      <c r="Q17" s="13" t="n">
         <v>14736</v>
       </c>
-      <c r="L17" s="13" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>21990</v>
-      </c>
-      <c r="N17" s="12" t="n">
+      <c r="R17" s="14" t="n">
+        <v>0.4102</v>
+      </c>
+      <c r="S17" s="13" t="n">
         <v>270885</v>
       </c>
-      <c r="O17" s="14" t="n">
+      <c r="T17" s="18" t="n">
         <v>1.67</v>
       </c>
-      <c r="P17" s="14" t="n">
+      <c r="U17" s="15" t="n">
         <v>1.56</v>
       </c>
-      <c r="Q17" s="14" t="n">
+      <c r="V17" s="15" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="W17" s="15" t="n">
         <v>0.11</v>
       </c>
-      <c r="R17" s="11" t="inlineStr"/>
-      <c r="S17" s="12" t="n">
+      <c r="X17" s="12" t="inlineStr"/>
+      <c r="Y17" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="T17" s="11" t="inlineStr">
+      <c r="Z17" s="12" t="inlineStr">
         <is>
           <t>🔧黒字転換+5,614(7/30判定)</t>
         </is>
       </c>
-      <c r="U17" s="15" t="inlineStr">
+      <c r="AA17" s="16" t="inlineStr">
         <is>
           <t>①7日利益 -5,129→+5,614に黒字転換＝複製リセットが効いた ②広告費率59.8%はまだ重い ③7/30判定。余裕+0.11と薄いので改善継続が条件 ④売価8,980円で値上げ余地は小さい(8.0%減まで)</t>
         </is>
@@ -2273,10 +2596,10 @@
       <c r="D18" s="5" t="n">
         <v>87075</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="19" t="n">
         <v>-22107</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="20" t="n">
         <v>-0.2195</v>
       </c>
       <c r="G18" s="8" t="n">
@@ -2285,69 +2608,85 @@
       <c r="H18" s="8" t="n">
         <v>0.8647</v>
       </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I18" s="5" t="n">
+        <v>45860</v>
       </c>
       <c r="J18" s="5" t="n">
+        <v>16055</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>34494</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>-4689</v>
+      </c>
+      <c r="M18" s="20" t="n">
+        <v>-0.1022</v>
+      </c>
+      <c r="N18" s="5" t="n">
         <v>13960</v>
       </c>
-      <c r="K18" s="17" t="n">
+      <c r="O18" s="5" t="n">
+        <v>5056</v>
+      </c>
+      <c r="P18" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="Q18" s="19" t="n">
         <v>-2096</v>
       </c>
-      <c r="L18" s="18" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="M18" s="17" t="n">
-        <v>-4689</v>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>105528</v>
-      </c>
-      <c r="O18" s="9" t="n">
+      <c r="R18" s="20" t="n">
+        <v>-0.1501</v>
+      </c>
+      <c r="S18" s="5" t="n">
+        <v>103812</v>
+      </c>
+      <c r="T18" s="18" t="n">
         <v>1.16</v>
       </c>
-      <c r="P18" s="9" t="n">
+      <c r="U18" s="10" t="n">
         <v>1.55</v>
       </c>
-      <c r="Q18" s="9" t="n">
+      <c r="V18" s="10" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="W18" s="10" t="n">
         <v>-0.39</v>
       </c>
-      <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="5" t="n">
+      <c r="X18" s="4" t="inlineStr"/>
+      <c r="Y18" s="5" t="n">
         <v>6000</v>
       </c>
-      <c r="T18" s="4" t="inlineStr">
+      <c r="Z18" s="4" t="inlineStr">
         <is>
           <t>🚨6kに半減済(8/1早期判定)</t>
         </is>
       </c>
-      <c r="U18" s="10" t="inlineStr">
+      <c r="AA18" s="11" t="inlineStr">
         <is>
           <t>①類似5%停止で6kに半減済。7/25消化11,000円は停止前の残り ②広告費率86.5%＝構造的に成立していない ③8/1にCPA&gt;6,000なら早期停止、8/6最終判定 ④週50CVに必要な44,887円/日は出せない</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>湯上がりガーゼワンピース</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <v>80720</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <v>27552</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <v>48535</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <v>4633</v>
       </c>
-      <c r="F19" s="16" t="n">
+      <c r="F19" s="17" t="n">
         <v>0.0574</v>
       </c>
       <c r="G19" s="8" t="n">
@@ -2356,43 +2695,59 @@
       <c r="H19" s="8" t="n">
         <v>0.6012999999999999</v>
       </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="19" t="n">
+      <c r="I19" s="13" t="n">
+        <v>5980</v>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>1968</v>
+      </c>
+      <c r="K19" s="13" t="n">
+        <v>17833</v>
+      </c>
+      <c r="L19" s="21" t="n">
+        <v>-13821</v>
+      </c>
+      <c r="M19" s="20" t="n">
+        <v>-2.3112</v>
+      </c>
+      <c r="N19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="13" t="n">
+        <v>5379</v>
+      </c>
+      <c r="Q19" s="21" t="n">
         <v>-5379</v>
       </c>
-      <c r="L19" s="11" t="inlineStr"/>
-      <c r="M19" s="19" t="n">
-        <v>-13821</v>
-      </c>
-      <c r="N19" s="12" t="n">
+      <c r="R19" s="12" t="inlineStr"/>
+      <c r="S19" s="13" t="n">
         <v>106500</v>
       </c>
-      <c r="O19" s="14" t="n">
+      <c r="T19" s="18" t="n">
         <v>1.66</v>
       </c>
-      <c r="P19" s="14" t="n">
+      <c r="U19" s="15" t="n">
         <v>1.52</v>
       </c>
-      <c r="Q19" s="14" t="n">
+      <c r="V19" s="15" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="W19" s="15" t="n">
         <v>0.14</v>
       </c>
-      <c r="R19" s="11" t="inlineStr"/>
-      <c r="S19" s="12" t="n">
+      <c r="X19" s="12" t="inlineStr"/>
+      <c r="Y19" s="13" t="n">
         <v>6500</v>
       </c>
-      <c r="T19" s="11" t="inlineStr">
+      <c r="Z19" s="12" t="inlineStr">
         <is>
           <t>🚨判定不合格(余裕+0.14&lt;+0.30)</t>
         </is>
       </c>
-      <c r="U19" s="15" t="inlineStr">
+      <c r="AA19" s="16" t="inlineStr">
         <is>
           <t>①★7/26判定で不合格（余裕+0.14 &lt; 基準+0.30）→停止 ②黒字転換はしたが日次利益662円と僅少、広告費率60.1% ③6,500円/日を4WAY(増分MER3.34)に回すと+7,668円/日＝11倍 ④夏物で9月以降の価値は低い</t>
         </is>
@@ -2416,7 +2771,7 @@
       <c r="E20" s="5" t="n">
         <v>6484</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F20" s="17" t="n">
         <v>0.0814</v>
       </c>
       <c r="G20" s="6" t="n">
@@ -2425,106 +2780,138 @@
       <c r="H20" s="8" t="n">
         <v>0.6568000000000001</v>
       </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I20" s="5" t="n">
+        <v>19920</v>
       </c>
       <c r="J20" s="5" t="n">
+        <v>5216</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>14589</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="M20" s="17" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="N20" s="5" t="n">
         <v>14940</v>
       </c>
-      <c r="K20" s="5" t="n">
+      <c r="O20" s="5" t="n">
+        <v>3912</v>
+      </c>
+      <c r="P20" s="5" t="n">
+        <v>4117</v>
+      </c>
+      <c r="Q20" s="5" t="n">
         <v>6911</v>
       </c>
-      <c r="L20" s="6" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>115</v>
-      </c>
-      <c r="N20" s="5" t="n">
+      <c r="R20" s="6" t="n">
+        <v>0.4626</v>
+      </c>
+      <c r="S20" s="5" t="n">
         <v>96139</v>
       </c>
-      <c r="O20" s="9" t="n">
+      <c r="T20" s="18" t="n">
         <v>1.52</v>
       </c>
-      <c r="P20" s="9" t="n">
+      <c r="U20" s="10" t="n">
         <v>1.35</v>
       </c>
-      <c r="Q20" s="9" t="n">
+      <c r="V20" s="10" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="W20" s="10" t="n">
         <v>0.17</v>
       </c>
-      <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="5" t="n">
+      <c r="X20" s="4" t="inlineStr"/>
+      <c r="Y20" s="5" t="n">
         <v>5000</v>
       </c>
-      <c r="T20" s="4" t="inlineStr">
+      <c r="Z20" s="4" t="inlineStr">
         <is>
           <t>🔧黒字+6,484(7/29判定)</t>
         </is>
       </c>
-      <c r="U20" s="10" t="inlineStr">
+      <c r="AA20" s="11" t="inlineStr">
         <is>
           <t>①7日利益+6,484、余裕+0.17 ②広告費率65.7%が主因、原価率26.2%は良好 ③増分MER0.00＝減らしても売上が落ちない。7/29判定で5k→3kも選択肢 ④非季節商品</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>瞬間冷却ハンディファン</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="13" t="n">
         <v>41860</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <v>14371</v>
       </c>
-      <c r="D21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12" t="n">
+      <c r="D21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="13" t="n">
         <v>27489</v>
       </c>
-      <c r="F21" s="13" t="n">
+      <c r="F21" s="14" t="n">
         <v>0.6567</v>
       </c>
       <c r="G21" s="8" t="n">
         <v>0.3433</v>
       </c>
-      <c r="H21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="11" t="inlineStr"/>
-      <c r="M21" s="12" t="n">
+      <c r="H21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>11960</v>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>4106</v>
+      </c>
+      <c r="K21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="13" t="n">
         <v>7854</v>
       </c>
-      <c r="N21" s="12" t="n">
+      <c r="M21" s="14" t="n">
+        <v>0.6567</v>
+      </c>
+      <c r="N21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="12" t="inlineStr"/>
+      <c r="S21" s="13" t="n">
         <v>70686</v>
       </c>
-      <c r="O21" s="11" t="inlineStr"/>
-      <c r="P21" s="11" t="inlineStr"/>
-      <c r="Q21" s="11" t="inlineStr"/>
-      <c r="R21" s="11" t="inlineStr"/>
-      <c r="S21" s="11" t="inlineStr"/>
-      <c r="T21" s="11" t="inlineStr">
+      <c r="T21" s="12" t="inlineStr"/>
+      <c r="U21" s="12" t="inlineStr"/>
+      <c r="V21" s="15" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="W21" s="12" t="inlineStr"/>
+      <c r="X21" s="12" t="inlineStr"/>
+      <c r="Y21" s="12" t="inlineStr"/>
+      <c r="Z21" s="12" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U21" s="15" t="inlineStr">
+      <c r="AA21" s="16" t="inlineStr">
         <is>
           <t>①広告ゼロで7日利益+33,264。4WAYからの流入 ②広告は出さない（4WAYと共食い） ③在庫消化用として現状維持</t>
         </is>
@@ -2557,98 +2944,130 @@
       <c r="H22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I22" s="5" t="n">
+        <v>15544</v>
       </c>
       <c r="J22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>15544</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="5" t="n">
         <v>3216</v>
       </c>
-      <c r="K22" s="5" t="n">
+      <c r="O22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="5" t="n">
         <v>3216</v>
       </c>
-      <c r="L22" s="6" t="n">
+      <c r="R22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M22" s="5" t="n">
-        <v>15544</v>
-      </c>
-      <c r="N22" s="5" t="n">
+      <c r="S22" s="5" t="n">
         <v>113632</v>
       </c>
-      <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
-      <c r="Q22" s="4" t="inlineStr"/>
-      <c r="R22" s="4" t="inlineStr"/>
-      <c r="S22" s="4" t="inlineStr"/>
-      <c r="T22" s="4" t="inlineStr">
+      <c r="T22" s="4" t="inlineStr"/>
+      <c r="U22" s="4" t="inlineStr"/>
+      <c r="V22" s="10" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="W22" s="4" t="inlineStr"/>
+      <c r="X22" s="4" t="inlineStr"/>
+      <c r="Y22" s="4" t="inlineStr"/>
+      <c r="Z22" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U22" s="10" t="inlineStr">
+      <c r="AA22" s="11" t="inlineStr">
         <is>
           <t>①7日75件/1,713注文＝アタッチ率4.38%（前週3.49%から改善） ②原価0＝売上全額が利益 ③15%到達で+141,156円/7日・利益率+0.94pt ④低単価帯(〜3,980円)のアタッチ率0%が最大の伸びしろ</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>完全遮光・接触冷感UVハット</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="13" t="n">
         <v>11960</v>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="13" t="n">
         <v>2822</v>
       </c>
-      <c r="D23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12" t="n">
+      <c r="D23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="13" t="n">
         <v>9138</v>
       </c>
-      <c r="F23" s="13" t="n">
+      <c r="F23" s="14" t="n">
         <v>0.764</v>
       </c>
-      <c r="G23" s="13" t="n">
+      <c r="G23" s="14" t="n">
         <v>0.236</v>
       </c>
-      <c r="H23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="11" t="inlineStr"/>
-      <c r="M23" s="12" t="n">
+      <c r="H23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="13" t="n">
+        <v>5980</v>
+      </c>
+      <c r="J23" s="13" t="n">
+        <v>1411</v>
+      </c>
+      <c r="K23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="13" t="n">
         <v>4569</v>
       </c>
-      <c r="N23" s="12" t="n">
+      <c r="M23" s="14" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="N23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="12" t="inlineStr"/>
+      <c r="S23" s="13" t="n">
         <v>41121</v>
       </c>
-      <c r="O23" s="11" t="inlineStr"/>
-      <c r="P23" s="11" t="inlineStr"/>
-      <c r="Q23" s="11" t="inlineStr"/>
-      <c r="R23" s="11" t="inlineStr"/>
-      <c r="S23" s="11" t="inlineStr"/>
-      <c r="T23" s="11" t="inlineStr">
+      <c r="T23" s="12" t="inlineStr"/>
+      <c r="U23" s="12" t="inlineStr"/>
+      <c r="V23" s="15" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="W23" s="12" t="inlineStr"/>
+      <c r="X23" s="12" t="inlineStr"/>
+      <c r="Y23" s="12" t="inlineStr"/>
+      <c r="Z23" s="12" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U23" s="15" t="inlineStr">
+      <c r="AA23" s="16" t="inlineStr">
         <is>
           <t>①広告ゼロ・利益率76.4% ②日傘/パーカーとのセット販売でクロスセルが本命 ③秋の帽子需要期(10月)に単独テスト候補</t>
         </is>
@@ -2681,10 +3100,8 @@
       <c r="H24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I24" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -2692,81 +3109,109 @@
       <c r="K24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="4" t="inlineStr"/>
-      <c r="M24" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr"/>
       <c r="N24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="4" t="inlineStr"/>
+      <c r="S24" s="5" t="n">
         <v>18697</v>
       </c>
-      <c r="O24" s="4" t="inlineStr"/>
-      <c r="P24" s="4" t="inlineStr"/>
-      <c r="Q24" s="4" t="inlineStr"/>
-      <c r="R24" s="4" t="inlineStr"/>
-      <c r="S24" s="4" t="inlineStr"/>
-      <c r="T24" s="4" t="inlineStr">
+      <c r="T24" s="4" t="inlineStr"/>
+      <c r="U24" s="4" t="inlineStr"/>
+      <c r="V24" s="10" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="W24" s="4" t="inlineStr"/>
+      <c r="X24" s="4" t="inlineStr"/>
+      <c r="Y24" s="4" t="inlineStr"/>
+      <c r="Z24" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U24" s="10" t="inlineStr">
+      <c r="AA24" s="11" t="inlineStr">
         <is>
           <t>①30日7個。8月で需要終了、今から出稿する価値なし ②来春(4月)のテスト枠候補</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>癒しの指圧マット</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="11" t="inlineStr"/>
-      <c r="G25" s="11" t="inlineStr"/>
-      <c r="H25" s="11" t="inlineStr"/>
-      <c r="I25" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="11" t="inlineStr"/>
-      <c r="M25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="12" t="n">
-        <v>4332</v>
-      </c>
-      <c r="O25" s="11" t="inlineStr"/>
-      <c r="P25" s="11" t="inlineStr"/>
-      <c r="Q25" s="11" t="inlineStr"/>
-      <c r="R25" s="11" t="inlineStr"/>
-      <c r="S25" s="11" t="inlineStr"/>
-      <c r="T25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>ネックマッサージャー</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="12" t="inlineStr"/>
+      <c r="G25" s="12" t="inlineStr"/>
+      <c r="H25" s="12" t="inlineStr"/>
+      <c r="I25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="12" t="inlineStr"/>
+      <c r="N25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="12" t="inlineStr"/>
+      <c r="S25" s="13" t="n">
+        <v>6946</v>
+      </c>
+      <c r="T25" s="12" t="inlineStr"/>
+      <c r="U25" s="12" t="inlineStr"/>
+      <c r="V25" s="12" t="inlineStr"/>
+      <c r="W25" s="12" t="inlineStr"/>
+      <c r="X25" s="12" t="inlineStr"/>
+      <c r="Y25" s="12" t="inlineStr"/>
+      <c r="Z25" s="12" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U25" s="15" t="inlineStr">
-        <is>
-          <t>①7/25改定で原価-262円と最大の値下げ、原価率27.6% ②秋冬の「おうち時間」需要でテスト枠候補</t>
+      <c r="AA25" s="16" t="inlineStr">
+        <is>
+          <t>①30日1個。売価9,980円・原価率30.4%は良好 ②秋冬需要（肩こり・ギフト）→11月テスト枠候補 ③今は何もしない</t>
         </is>
       </c>
     </row>
@@ -2791,10 +3236,8 @@
       <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="4" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I26" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0</v>
@@ -2802,88 +3245,114 @@
       <c r="K26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4" t="inlineStr"/>
       <c r="N26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="4" t="inlineStr"/>
+      <c r="S26" s="5" t="n">
         <v>4551</v>
       </c>
-      <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="4" t="inlineStr"/>
-      <c r="Q26" s="4" t="inlineStr"/>
-      <c r="R26" s="4" t="inlineStr"/>
-      <c r="S26" s="4" t="inlineStr"/>
-      <c r="T26" s="4" t="inlineStr">
+      <c r="T26" s="4" t="inlineStr"/>
+      <c r="U26" s="4" t="inlineStr"/>
+      <c r="V26" s="4" t="inlineStr"/>
+      <c r="W26" s="4" t="inlineStr"/>
+      <c r="X26" s="4" t="inlineStr"/>
+      <c r="Y26" s="4" t="inlineStr"/>
+      <c r="Z26" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U26" s="10" t="inlineStr">
+      <c r="AA26" s="11" t="inlineStr">
         <is>
           <t>①30日1個。原価率24.1%は良好だが需要が立っていない ②在庫リスクなし、放置で可</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>ナノバブルシャワーヘッド</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="11" t="inlineStr"/>
-      <c r="G27" s="11" t="inlineStr"/>
-      <c r="H27" s="11" t="inlineStr"/>
-      <c r="I27" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="J27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="11" t="inlineStr"/>
-      <c r="M27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>51975</v>
-      </c>
-      <c r="O27" s="11" t="inlineStr"/>
-      <c r="P27" s="11" t="inlineStr"/>
-      <c r="Q27" s="11" t="inlineStr"/>
-      <c r="R27" s="11" t="inlineStr"/>
-      <c r="S27" s="11" t="inlineStr"/>
-      <c r="T27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>癒しの指圧マット</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="12" t="inlineStr"/>
+      <c r="G27" s="12" t="inlineStr"/>
+      <c r="H27" s="12" t="inlineStr"/>
+      <c r="I27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="12" t="inlineStr"/>
+      <c r="N27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="12" t="inlineStr"/>
+      <c r="S27" s="13" t="n">
+        <v>4332</v>
+      </c>
+      <c r="T27" s="12" t="inlineStr"/>
+      <c r="U27" s="12" t="inlineStr"/>
+      <c r="V27" s="12" t="inlineStr"/>
+      <c r="W27" s="12" t="inlineStr"/>
+      <c r="X27" s="12" t="inlineStr"/>
+      <c r="Y27" s="12" t="inlineStr"/>
+      <c r="Z27" s="12" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U27" s="15" t="inlineStr">
-        <is>
-          <t>①30日7.7万円・広告ゼロ。原価率32.3%・分岐MER1.48 ②秋冬に需要増（入浴時間の増加） ③9月のテスト枠の第一候補</t>
+      <c r="AA27" s="16" t="inlineStr">
+        <is>
+          <t>①7/25改定で原価-262円と最大の値下げ、原価率27.6% ②秋冬の「おうち時間」需要でテスト枠候補</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>ネックマッサージャー</t>
+          <t>ナノバブルシャワーヘッド</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
@@ -2901,10 +3370,8 @@
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
+      <c r="I28" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0</v>
@@ -2912,26 +3379,40 @@
       <c r="K28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L28" s="4" t="inlineStr"/>
-      <c r="M28" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="4" t="inlineStr"/>
       <c r="N28" s="5" t="n">
-        <v>6946</v>
-      </c>
-      <c r="O28" s="4" t="inlineStr"/>
-      <c r="P28" s="4" t="inlineStr"/>
-      <c r="Q28" s="4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="O28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="R28" s="4" t="inlineStr"/>
-      <c r="S28" s="4" t="inlineStr"/>
-      <c r="T28" s="4" t="inlineStr">
+      <c r="S28" s="5" t="n">
+        <v>51975</v>
+      </c>
+      <c r="T28" s="4" t="inlineStr"/>
+      <c r="U28" s="4" t="inlineStr"/>
+      <c r="V28" s="4" t="inlineStr"/>
+      <c r="W28" s="4" t="inlineStr"/>
+      <c r="X28" s="4" t="inlineStr"/>
+      <c r="Y28" s="4" t="inlineStr"/>
+      <c r="Z28" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="U28" s="10" t="inlineStr">
-        <is>
-          <t>①30日1個。売価9,980円・原価率30.4%は良好 ②秋冬需要（肩こり・ギフト）→11月テスト枠候補 ③今は何もしない</t>
+      <c r="AA28" s="11" t="inlineStr">
+        <is>
+          <t>①30日7.7万円・広告ゼロ。原価率32.3%・分岐MER1.48 ②秋冬に需要増（入浴時間の増加） ③9月のテスト枠の第一候補</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document why MER drives the decisions, and format the headline numbers
MER is not a more accurate ROAS — it divides measured Shopify revenue by
spend, where ROAS divides Meta's attributed value. Record the reasoning as
section 6b so every report carries it: margin ties to MER algebraically,
Meta's per-product attribution swings 79-108%, the platform grades its own
work, and MER's denominator catches unallocatable catalog spend.

Also note MER's weakness — non-ad revenue sits in its numerator — and that
incremental MER is what covers it.

Headline comparison figures now render with thousands separators.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-26.xlsx
+++ b/data/reports/report-2026-07-26.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +126,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -512,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -583,19 +586,19 @@
           <t>売上(gross−値引)</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>1379567</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>1311185</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>1390938</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>1442194</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>1285330</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -610,17 +613,17 @@
           <t>原価</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>413436</v>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>419409</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>439144</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="5" t="n">
         <v>373455</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -635,17 +638,17 @@
           <t>広告費</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>555701</v>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>552400</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>545552</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="5" t="n">
         <v>463968</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -660,17 +663,17 @@
           <t>利益</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>410430</v>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>419130</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="5" t="n">
         <v>457498</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="5" t="n">
         <v>447908</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -718,17 +721,17 @@
           <t>手数料控除後利益</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <v>362283</v>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <v>370586</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <v>407165</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="5" t="n">
         <v>403050</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -797,28 +800,28 @@
           <t>前日(7/25 土)</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <v>1379567</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>413436</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="6" t="n">
         <v>555701</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="6" t="n">
         <v>410430</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="7" t="n">
         <v>0.298</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="6" t="n">
         <v>48147</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="6" t="n">
         <v>362283</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="7" t="n">
         <v>0.263</v>
       </c>
     </row>
@@ -828,28 +831,28 @@
           <t>3日(7/23-25)</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <v>4172815</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <v>1258227</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="6" t="n">
         <v>1657199</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
         <v>1257389</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="7" t="n">
         <v>0.301</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="6" t="n">
         <v>145631</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="6" t="n">
         <v>1111758</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="7" t="n">
         <v>0.266</v>
       </c>
     </row>
@@ -859,28 +862,28 @@
           <t>7日(7/19-25)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="6" t="n">
         <v>10095358</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="6" t="n">
         <v>3074011</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="6" t="n">
         <v>3818861</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="6" t="n">
         <v>3202486</v>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="7" t="n">
         <v>0.317</v>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="G16" s="6" t="n">
         <v>352328</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="H16" s="6" t="n">
         <v>2850158</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="7" t="n">
         <v>0.282</v>
       </c>
     </row>
@@ -890,28 +893,28 @@
           <t>30日(6/26-7/25)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="6" t="n">
         <v>38559901</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="6" t="n">
         <v>11203519</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="6" t="n">
         <v>13919026</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="6" t="n">
         <v>13437356</v>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="7" t="n">
         <v>0.348</v>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="6" t="n">
         <v>1345741</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="H17" s="6" t="n">
         <v>12091615</v>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="I17" s="7" t="n">
         <v>0.314</v>
       </c>
     </row>
@@ -921,89 +924,103 @@
           <t>📅7/18〜7/25累積(8日)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="6" t="n">
         <v>11417483</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="6" t="n">
         <v>3448948</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="6" t="n">
         <v>4321489</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="6" t="n">
         <v>3647046</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F18" s="7" t="n">
         <v>0.319</v>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="G18" s="6" t="n">
         <v>398470</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H18" s="6" t="n">
         <v>3248576</v>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I18" s="7" t="n">
         <v>0.285</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>・売上=gross_sales−discounts（返品A案）。当月返品累計 7/25時点 187,481円（返品率0.58%）。7/25 新規返品ゼロ</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>・★判断軸がMERである理由: ①利益率=1−原価率−1/MER で数式が直結する ②商品別のMeta計上は突合率79〜108%とブレる（4WAY79%・サンダル79%・スリッパ108%）③Metaの数値は媒体の自己申告 ④カタログ広告など商品配賦できない費用も分母に入り帳尻が合う</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>・★MERは「正確なROAS」ではなく別物。ROAS=Meta計上値(推定)÷広告費、MER=Shopify実売上(実測)÷広告費。MERは非広告流入も分子に含むため広告の貢献を過大評価する（7日実測でMetaは全店売上の96%を計上、非広告分は約4%=385,277円）。この弱点を埋めるのが増分MERで、MER=継続/停止の判定、増分MER=予算増減の判定と使い分ける</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>・★列を「7日 → 3日 → 前日」の順に並べ替え、3日も売上/原価/広告費/利益/利益率の5項目に拡張（前日も同じ5項目に統一）</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>・★目標MER列を追加。目標MER = 1 ÷ (1 − その商品の原価率 − 0.35)。商品ごとに2.17〜5.49と差が大きいため全店値2.91は使わない。MER列は目標超え=緑・未達=赤</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>・★3日利益率は全商品に表示（従来は日販20個以上に限定）。ただし日販10個未満の商品は日次のブレが13〜64ptあり、3日平均でも実力を測れない点は変わらない</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>・★7/26判定: 湯上がりガーゼワンピースは7日余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>・★増額候補（自分の目標MER超え×消化率95%以上）: 害虫ブロッカー(2.78&gt;2.31・102%)・ナノガラス脱毛パッド(2.39&gt;2.17・100%)・完全遮光(2.70&gt;2.56・95%)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>・全期間の広告費・原価はMeta/Shopifyの実測。推計・外挿は不使用</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>・30日窓の途中開始: 卓上冷感クーラー7/13(13日)・5WAY腰掛けファン7/19(7日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10(16日)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>・増分MER: 7/22以降に予算を3,000円/日以上動かした商品がないため全商品「判定保留」</t>
         </is>
@@ -1195,74 +1212,74 @@
           <t>4WAY 取り付けOK 小型瞬間冷却ハンディファン</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="6" t="n">
         <v>2245980</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="6" t="n">
         <v>780230</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="6" t="n">
         <v>569994</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="6" t="n">
         <v>895756</v>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="F2" s="7" t="n">
         <v>0.3988</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="9" t="n">
         <v>0.3474</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="7" t="n">
         <v>0.2538</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="6" t="n">
         <v>976080</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="6" t="n">
         <v>339080</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="6" t="n">
         <v>259502</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="6" t="n">
         <v>377498</v>
       </c>
-      <c r="M2" s="6" t="n">
+      <c r="M2" s="7" t="n">
         <v>0.3867</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="N2" s="6" t="n">
         <v>348600</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="O2" s="6" t="n">
         <v>121100</v>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="P2" s="6" t="n">
         <v>87318</v>
       </c>
-      <c r="Q2" s="5" t="n">
+      <c r="Q2" s="6" t="n">
         <v>140182</v>
       </c>
-      <c r="R2" s="6" t="n">
+      <c r="R2" s="7" t="n">
         <v>0.4021</v>
       </c>
-      <c r="S2" s="5" t="n">
+      <c r="S2" s="6" t="n">
         <v>2697046</v>
       </c>
-      <c r="T2" s="9" t="n">
+      <c r="T2" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="U2" s="10" t="n">
+      <c r="U2" s="11" t="n">
         <v>1.53</v>
       </c>
-      <c r="V2" s="10" t="n">
+      <c r="V2" s="11" t="n">
         <v>3.3</v>
       </c>
-      <c r="W2" s="10" t="n">
+      <c r="W2" s="11" t="n">
         <v>2.41</v>
       </c>
       <c r="X2" s="4" t="inlineStr"/>
-      <c r="Y2" s="5" t="n">
+      <c r="Y2" s="6" t="n">
         <v>95000</v>
       </c>
       <c r="Z2" s="4" t="inlineStr">
@@ -1270,94 +1287,94 @@
           <t>✅95k初日(7/28判定)</t>
         </is>
       </c>
-      <c r="AA2" s="11" t="inlineStr">
+      <c r="AA2" s="12" t="inlineStr">
         <is>
           <t>①7/25に95kへ増額。消化率90%で余裕あり→7/28に増分MER≥2.91なら110k ②原価率34.7%。月1,344個の最大SKU＝CJ数量交渉の最有力 ③+500円値上げは13.3%減まで許容</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>形状記憶日傘</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="14" t="n">
         <v>1439220</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="14" t="n">
         <v>378301</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="14" t="n">
         <v>419790</v>
       </c>
-      <c r="E3" s="13" t="n">
+      <c r="E3" s="14" t="n">
         <v>641129</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="F3" s="15" t="n">
         <v>0.4455</v>
       </c>
-      <c r="G3" s="14" t="n">
+      <c r="G3" s="15" t="n">
         <v>0.2629</v>
       </c>
-      <c r="H3" s="14" t="n">
+      <c r="H3" s="15" t="n">
         <v>0.2917</v>
       </c>
-      <c r="I3" s="13" t="n">
+      <c r="I3" s="14" t="n">
         <v>537840</v>
       </c>
-      <c r="J3" s="13" t="n">
+      <c r="J3" s="14" t="n">
         <v>141372</v>
       </c>
-      <c r="K3" s="13" t="n">
+      <c r="K3" s="14" t="n">
         <v>168540</v>
       </c>
-      <c r="L3" s="13" t="n">
+      <c r="L3" s="14" t="n">
         <v>227928</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="M3" s="15" t="n">
         <v>0.4238</v>
       </c>
-      <c r="N3" s="13" t="n">
+      <c r="N3" s="14" t="n">
         <v>219120</v>
       </c>
-      <c r="O3" s="13" t="n">
+      <c r="O3" s="14" t="n">
         <v>57596</v>
       </c>
-      <c r="P3" s="13" t="n">
+      <c r="P3" s="14" t="n">
         <v>54689</v>
       </c>
-      <c r="Q3" s="13" t="n">
+      <c r="Q3" s="14" t="n">
         <v>106835</v>
       </c>
-      <c r="R3" s="14" t="n">
+      <c r="R3" s="15" t="n">
         <v>0.4876</v>
       </c>
-      <c r="S3" s="13" t="n">
+      <c r="S3" s="14" t="n">
         <v>2127799</v>
       </c>
-      <c r="T3" s="9" t="n">
+      <c r="T3" s="10" t="n">
         <v>3.43</v>
       </c>
-      <c r="U3" s="15" t="n">
+      <c r="U3" s="16" t="n">
         <v>1.36</v>
       </c>
-      <c r="V3" s="15" t="n">
+      <c r="V3" s="16" t="n">
         <v>2.58</v>
       </c>
-      <c r="W3" s="15" t="n">
+      <c r="W3" s="16" t="n">
         <v>2.07</v>
       </c>
-      <c r="X3" s="12" t="inlineStr"/>
-      <c r="Y3" s="13" t="n">
+      <c r="X3" s="13" t="inlineStr"/>
+      <c r="Y3" s="14" t="n">
         <v>60000</v>
       </c>
-      <c r="Z3" s="12" t="inlineStr">
+      <c r="Z3" s="13" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="AA3" s="16" t="inlineStr">
+      <c r="AA3" s="17" t="inlineStr">
         <is>
           <t>①MER3.43・余裕+2.07に改善、消化率93%。据置 ②原価率26.3%・広告費率29.2%とも健全 ③お盆明け(8/15)から段階減額の計画を</t>
         </is>
@@ -1369,74 +1386,74 @@
           <t>害虫ブロッカー</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="6" t="n">
         <v>1400960</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="6" t="n">
         <v>304317</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="6" t="n">
         <v>503299</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="6" t="n">
         <v>593344</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="7" t="n">
         <v>0.4235</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="7" t="n">
         <v>0.2172</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="7" t="n">
         <v>0.3593</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="6" t="n">
         <v>589040</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="6" t="n">
         <v>128316</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="6" t="n">
         <v>220153</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="6" t="n">
         <v>240571</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="M4" s="7" t="n">
         <v>0.4084</v>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="N4" s="6" t="n">
         <v>199000</v>
       </c>
-      <c r="O4" s="5" t="n">
+      <c r="O4" s="6" t="n">
         <v>43350</v>
       </c>
-      <c r="P4" s="5" t="n">
+      <c r="P4" s="6" t="n">
         <v>77160</v>
       </c>
-      <c r="Q4" s="5" t="n">
+      <c r="Q4" s="6" t="n">
         <v>78490</v>
       </c>
-      <c r="R4" s="6" t="n">
+      <c r="R4" s="7" t="n">
         <v>0.3944</v>
       </c>
-      <c r="S4" s="5" t="n">
+      <c r="S4" s="6" t="n">
         <v>3921630</v>
       </c>
-      <c r="T4" s="9" t="n">
+      <c r="T4" s="10" t="n">
         <v>2.78</v>
       </c>
-      <c r="U4" s="10" t="n">
+      <c r="U4" s="11" t="n">
         <v>1.28</v>
       </c>
-      <c r="V4" s="10" t="n">
+      <c r="V4" s="11" t="n">
         <v>2.31</v>
       </c>
-      <c r="W4" s="10" t="n">
+      <c r="W4" s="11" t="n">
         <v>1.5</v>
       </c>
       <c r="X4" s="4" t="inlineStr"/>
-      <c r="Y4" s="5" t="n">
+      <c r="Y4" s="6" t="n">
         <v>73000</v>
       </c>
       <c r="Z4" s="4" t="inlineStr">
@@ -1444,94 +1461,94 @@
           <t>✅維持</t>
         </is>
       </c>
-      <c r="AA4" s="11" t="inlineStr">
+      <c r="AA4" s="12" t="inlineStr">
         <is>
           <t>①消化率102%で天井張り付き。ただしMER2.78&lt;目標2.91＝増額は率を薄める。据置 ②原価率21.7%は最良 ③30日利益の最大の稼ぎ頭。触らないのが最善</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>ナノガラス脱毛パッド</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="14" t="n">
         <v>899480</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>169773</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>376745</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="14" t="n">
         <v>352962</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="15" t="n">
         <v>0.3924</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="15" t="n">
         <v>0.1887</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="9" t="n">
         <v>0.4188</v>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="14" t="n">
         <v>398000</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="14" t="n">
         <v>75105</v>
       </c>
-      <c r="K5" s="13" t="n">
+      <c r="K5" s="14" t="n">
         <v>175607</v>
       </c>
-      <c r="L5" s="13" t="n">
+      <c r="L5" s="14" t="n">
         <v>147288</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="M5" s="15" t="n">
         <v>0.3701</v>
       </c>
-      <c r="N5" s="13" t="n">
+      <c r="N5" s="14" t="n">
         <v>163180</v>
       </c>
-      <c r="O5" s="13" t="n">
+      <c r="O5" s="14" t="n">
         <v>30782</v>
       </c>
-      <c r="P5" s="13" t="n">
+      <c r="P5" s="14" t="n">
         <v>61455</v>
       </c>
-      <c r="Q5" s="13" t="n">
+      <c r="Q5" s="14" t="n">
         <v>70943</v>
       </c>
-      <c r="R5" s="14" t="n">
+      <c r="R5" s="15" t="n">
         <v>0.4348</v>
       </c>
-      <c r="S5" s="13" t="n">
+      <c r="S5" s="14" t="n">
         <v>2241388</v>
       </c>
-      <c r="T5" s="9" t="n">
+      <c r="T5" s="10" t="n">
         <v>2.39</v>
       </c>
-      <c r="U5" s="15" t="n">
+      <c r="U5" s="16" t="n">
         <v>1.23</v>
       </c>
-      <c r="V5" s="15" t="n">
+      <c r="V5" s="16" t="n">
         <v>2.17</v>
       </c>
-      <c r="W5" s="15" t="n">
+      <c r="W5" s="16" t="n">
         <v>1.16</v>
       </c>
-      <c r="X5" s="12" t="inlineStr"/>
-      <c r="Y5" s="13" t="n">
+      <c r="X5" s="13" t="inlineStr"/>
+      <c r="Y5" s="14" t="n">
         <v>60000</v>
       </c>
-      <c r="Z5" s="12" t="inlineStr">
+      <c r="Z5" s="13" t="inlineStr">
         <is>
           <t>✅BC検証中</t>
         </is>
       </c>
-      <c r="AA5" s="16" t="inlineStr">
+      <c r="AA5" s="17" t="inlineStr">
         <is>
           <t>①消化率100%天井だが余裕+1.15・MER2.39と目標未達。BC検証の結果待ち ②原価率18.9%は全商品最良、広告費率41.9%が重し ③通年需要＝秋以降の主力候補</t>
         </is>
@@ -1543,74 +1560,74 @@
           <t>卓上冷感クーラー</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>771420</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="n">
         <v>257484</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="6" t="n">
         <v>195416</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="6" t="n">
         <v>318520</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <v>0.4129</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <v>0.3338</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="7" t="n">
         <v>0.2533</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="6" t="n">
         <v>334880</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="6" t="n">
         <v>111776</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="6" t="n">
         <v>95579</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L6" s="6" t="n">
         <v>127525</v>
       </c>
-      <c r="M6" s="6" t="n">
+      <c r="M6" s="7" t="n">
         <v>0.3808</v>
       </c>
-      <c r="N6" s="5" t="n">
+      <c r="N6" s="6" t="n">
         <v>53820</v>
       </c>
-      <c r="O6" s="5" t="n">
+      <c r="O6" s="6" t="n">
         <v>17964</v>
       </c>
-      <c r="P6" s="5" t="n">
+      <c r="P6" s="6" t="n">
         <v>35525</v>
       </c>
-      <c r="Q6" s="5" t="n">
+      <c r="Q6" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="R6" s="17" t="n">
+      <c r="R6" s="18" t="n">
         <v>0.0062</v>
       </c>
-      <c r="S6" s="5" t="n">
+      <c r="S6" s="6" t="n">
         <v>472286</v>
       </c>
-      <c r="T6" s="9" t="n">
+      <c r="T6" s="10" t="n">
         <v>3.95</v>
       </c>
-      <c r="U6" s="10" t="n">
+      <c r="U6" s="11" t="n">
         <v>1.5</v>
       </c>
-      <c r="V6" s="10" t="n">
+      <c r="V6" s="11" t="n">
         <v>3.16</v>
       </c>
-      <c r="W6" s="10" t="n">
+      <c r="W6" s="11" t="n">
         <v>2.45</v>
       </c>
       <c r="X6" s="4" t="inlineStr"/>
-      <c r="Y6" s="5" t="n">
+      <c r="Y6" s="6" t="n">
         <v>38000</v>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -1618,94 +1635,94 @@
           <t>✅消化率88%回復(7/27判定)</t>
         </is>
       </c>
-      <c r="AA6" s="11" t="inlineStr">
+      <c r="AA6" s="12" t="inlineStr">
         <is>
           <t>①消化率79%→88%に回復。7/27に増分MER判定 ②原価率33.4%。+500円値上げは11.2%減まで許容 ③MER3.95・余裕+2.45と好調</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>完全遮光・形状記憶・晴雨兼用・UV日傘</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>702180</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>181951</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>260052</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="14" t="n">
         <v>260177</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="15" t="n">
         <v>0.3705</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="15" t="n">
         <v>0.2591</v>
       </c>
-      <c r="H7" s="14" t="n">
+      <c r="H7" s="15" t="n">
         <v>0.3703</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="14" t="n">
         <v>268920</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="14" t="n">
         <v>69377</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K7" s="14" t="n">
         <v>117885</v>
       </c>
-      <c r="L7" s="13" t="n">
+      <c r="L7" s="14" t="n">
         <v>81658</v>
       </c>
-      <c r="M7" s="14" t="n">
+      <c r="M7" s="15" t="n">
         <v>0.3037</v>
       </c>
-      <c r="N7" s="13" t="n">
+      <c r="N7" s="14" t="n">
         <v>49800</v>
       </c>
-      <c r="O7" s="13" t="n">
+      <c r="O7" s="14" t="n">
         <v>11781</v>
       </c>
-      <c r="P7" s="13" t="n">
+      <c r="P7" s="14" t="n">
         <v>37609</v>
       </c>
-      <c r="Q7" s="13" t="n">
+      <c r="Q7" s="14" t="n">
         <v>410</v>
       </c>
-      <c r="R7" s="17" t="n">
+      <c r="R7" s="18" t="n">
         <v>0.008200000000000001</v>
       </c>
-      <c r="S7" s="13" t="n">
+      <c r="S7" s="14" t="n">
         <v>916606</v>
       </c>
-      <c r="T7" s="9" t="n">
+      <c r="T7" s="10" t="n">
         <v>2.7</v>
       </c>
-      <c r="U7" s="15" t="n">
+      <c r="U7" s="16" t="n">
         <v>1.35</v>
       </c>
-      <c r="V7" s="15" t="n">
+      <c r="V7" s="16" t="n">
         <v>2.56</v>
       </c>
-      <c r="W7" s="15" t="n">
+      <c r="W7" s="16" t="n">
         <v>1.35</v>
       </c>
-      <c r="X7" s="12" t="inlineStr"/>
-      <c r="Y7" s="13" t="n">
+      <c r="X7" s="13" t="inlineStr"/>
+      <c r="Y7" s="14" t="n">
         <v>41000</v>
       </c>
-      <c r="Z7" s="12" t="inlineStr">
+      <c r="Z7" s="13" t="inlineStr">
         <is>
           <t>👀余裕+1.35(7/28判定)</t>
         </is>
       </c>
-      <c r="AA7" s="16" t="inlineStr">
+      <c r="AA7" s="17" t="inlineStr">
         <is>
           <t>①余裕+1.82→+1.35に低下、MER3.17→2.70。7/28判定で増分MER&lt;2.91なら据置確定 ②日傘2本合算MER3.20 ③8/15から減額</t>
         </is>
@@ -1717,74 +1734,74 @@
           <t>接触冷感UVパーカー</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>616900</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
         <v>222270</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="6" t="n">
         <v>216551</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
         <v>178079</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="18" t="n">
         <v>0.2887</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <v>0.3603</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="7" t="n">
         <v>0.351</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="6" t="n">
         <v>290540</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="6" t="n">
         <v>104682</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="6" t="n">
         <v>98985</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="L8" s="6" t="n">
         <v>86873</v>
       </c>
-      <c r="M8" s="17" t="n">
+      <c r="M8" s="18" t="n">
         <v>0.299</v>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="N8" s="6" t="n">
         <v>83580</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="O8" s="6" t="n">
         <v>30114</v>
       </c>
-      <c r="P8" s="5" t="n">
+      <c r="P8" s="6" t="n">
         <v>34385</v>
       </c>
-      <c r="Q8" s="5" t="n">
+      <c r="Q8" s="6" t="n">
         <v>19081</v>
       </c>
-      <c r="R8" s="17" t="n">
+      <c r="R8" s="18" t="n">
         <v>0.2283</v>
       </c>
-      <c r="S8" s="5" t="n">
+      <c r="S8" s="6" t="n">
         <v>760675</v>
       </c>
-      <c r="T8" s="18" t="n">
+      <c r="T8" s="19" t="n">
         <v>2.85</v>
       </c>
-      <c r="U8" s="10" t="n">
+      <c r="U8" s="11" t="n">
         <v>1.56</v>
       </c>
-      <c r="V8" s="10" t="n">
+      <c r="V8" s="11" t="n">
         <v>3.45</v>
       </c>
-      <c r="W8" s="10" t="n">
+      <c r="W8" s="11" t="n">
         <v>1.29</v>
       </c>
       <c r="X8" s="4" t="inlineStr"/>
-      <c r="Y8" s="5" t="n">
+      <c r="Y8" s="6" t="n">
         <v>34000</v>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1792,94 +1809,94 @@
           <t>⚠️利益率28.9%(7/28判定)</t>
         </is>
       </c>
-      <c r="AA8" s="11" t="inlineStr">
+      <c r="AA8" s="12" t="inlineStr">
         <is>
           <t>①利益率35.0%→28.9%に悪化、消化率98%天井。7/28判定 ②原価率36.0%。売価3,980円で+500円値上げは16.4%減まで許容＝値上げ余地最大 ③CR疲弊の可能性→素材があれば投入</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>5WAY腰掛けファン</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <v>393420</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>145992</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>76449</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="14" t="n">
         <v>170979</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>0.4346</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>0.3711</v>
       </c>
-      <c r="H9" s="14" t="n">
+      <c r="H9" s="15" t="n">
         <v>0.1943</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="I9" s="14" t="n">
         <v>144420</v>
       </c>
-      <c r="J9" s="13" t="n">
+      <c r="J9" s="14" t="n">
         <v>53592</v>
       </c>
-      <c r="K9" s="13" t="n">
+      <c r="K9" s="14" t="n">
         <v>36556</v>
       </c>
-      <c r="L9" s="13" t="n">
+      <c r="L9" s="14" t="n">
         <v>54272</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="M9" s="15" t="n">
         <v>0.3758</v>
       </c>
-      <c r="N9" s="13" t="n">
+      <c r="N9" s="14" t="n">
         <v>59760</v>
       </c>
-      <c r="O9" s="13" t="n">
+      <c r="O9" s="14" t="n">
         <v>22176</v>
       </c>
-      <c r="P9" s="13" t="n">
+      <c r="P9" s="14" t="n">
         <v>12036</v>
       </c>
-      <c r="Q9" s="13" t="n">
+      <c r="Q9" s="14" t="n">
         <v>25548</v>
       </c>
-      <c r="R9" s="14" t="n">
+      <c r="R9" s="15" t="n">
         <v>0.4275</v>
       </c>
-      <c r="S9" s="13" t="n">
+      <c r="S9" s="14" t="n">
         <v>170979</v>
       </c>
-      <c r="T9" s="9" t="n">
+      <c r="T9" s="10" t="n">
         <v>5.15</v>
       </c>
-      <c r="U9" s="15" t="n">
+      <c r="U9" s="16" t="n">
         <v>1.59</v>
       </c>
-      <c r="V9" s="15" t="n">
+      <c r="V9" s="16" t="n">
         <v>3.59</v>
       </c>
-      <c r="W9" s="15" t="n">
+      <c r="W9" s="16" t="n">
         <v>3.56</v>
       </c>
-      <c r="X9" s="12" t="inlineStr"/>
-      <c r="Y9" s="13" t="n">
+      <c r="X9" s="13" t="inlineStr"/>
+      <c r="Y9" s="14" t="n">
         <v>13000</v>
       </c>
-      <c r="Z9" s="12" t="inlineStr">
+      <c r="Z9" s="13" t="inlineStr">
         <is>
           <t>👀学習中(7/28判定)</t>
         </is>
       </c>
-      <c r="AA9" s="16" t="inlineStr">
+      <c r="AA9" s="17" t="inlineStr">
         <is>
           <t>①MER5.15・余裕+3.56で全商品最高効率。消化率92% ②広告費率19.4%は最良＝伸びしろ最大。7/28判定で増額候補 ③原価率37.1%が唯一の弱点</t>
         </is>
@@ -1891,74 +1908,74 @@
           <t>3WAYサーキュレーター扇風機</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>304980</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>126735</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="6" t="n">
         <v>101952</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="6" t="n">
         <v>76293</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="18" t="n">
         <v>0.2502</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="9" t="n">
         <v>0.4156</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="7" t="n">
         <v>0.3343</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="6" t="n">
         <v>71760</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="6" t="n">
         <v>29820</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="6" t="n">
         <v>46807</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="L10" s="20" t="n">
         <v>-4867</v>
       </c>
-      <c r="M10" s="20" t="n">
+      <c r="M10" s="21" t="n">
         <v>-0.0678</v>
       </c>
-      <c r="N10" s="5" t="n">
+      <c r="N10" s="6" t="n">
         <v>17940</v>
       </c>
-      <c r="O10" s="5" t="n">
+      <c r="O10" s="6" t="n">
         <v>7455</v>
       </c>
-      <c r="P10" s="5" t="n">
+      <c r="P10" s="6" t="n">
         <v>16363</v>
       </c>
-      <c r="Q10" s="19" t="n">
+      <c r="Q10" s="20" t="n">
         <v>-5878</v>
       </c>
-      <c r="R10" s="20" t="n">
+      <c r="R10" s="21" t="n">
         <v>-0.3276</v>
       </c>
-      <c r="S10" s="5" t="n">
+      <c r="S10" s="6" t="n">
         <v>218247</v>
       </c>
-      <c r="T10" s="18" t="n">
+      <c r="T10" s="19" t="n">
         <v>2.99</v>
       </c>
-      <c r="U10" s="10" t="n">
+      <c r="U10" s="11" t="n">
         <v>1.71</v>
       </c>
-      <c r="V10" s="10" t="n">
+      <c r="V10" s="11" t="n">
         <v>4.27</v>
       </c>
-      <c r="W10" s="10" t="n">
+      <c r="W10" s="11" t="n">
         <v>1.28</v>
       </c>
       <c r="X10" s="4" t="inlineStr"/>
-      <c r="Y10" s="5" t="n">
+      <c r="Y10" s="6" t="n">
         <v>16000</v>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1966,94 +1983,94 @@
           <t>✅維持</t>
         </is>
       </c>
-      <c r="AA10" s="11" t="inlineStr">
+      <c r="AA10" s="12" t="inlineStr">
         <is>
           <t>①消化率101%天井・MER2.99。据置 ②原価率41.6%が主因で利益率25.0% ③5,980→6,980円の値上げは22.2%減まで許容＝値上げ最有力 ④CJ交渉で2,485→2,200円なら利益率+4.8pt</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>偏光・調光サングラス</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="14" t="n">
         <v>266660</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>59831</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>153852</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <v>52977</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="F11" s="18" t="n">
         <v>0.1987</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G11" s="15" t="n">
         <v>0.2244</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="9" t="n">
         <v>0.577</v>
       </c>
-      <c r="I11" s="13" t="n">
+      <c r="I11" s="14" t="n">
         <v>99500</v>
       </c>
-      <c r="J11" s="13" t="n">
+      <c r="J11" s="14" t="n">
         <v>22325</v>
       </c>
-      <c r="K11" s="13" t="n">
+      <c r="K11" s="14" t="n">
         <v>61213</v>
       </c>
-      <c r="L11" s="13" t="n">
+      <c r="L11" s="14" t="n">
         <v>15962</v>
       </c>
-      <c r="M11" s="17" t="n">
+      <c r="M11" s="18" t="n">
         <v>0.1604</v>
       </c>
-      <c r="N11" s="13" t="n">
+      <c r="N11" s="14" t="n">
         <v>19900</v>
       </c>
-      <c r="O11" s="13" t="n">
+      <c r="O11" s="14" t="n">
         <v>4465</v>
       </c>
-      <c r="P11" s="13" t="n">
+      <c r="P11" s="14" t="n">
         <v>19381</v>
       </c>
-      <c r="Q11" s="21" t="n">
+      <c r="Q11" s="22" t="n">
         <v>-3946</v>
       </c>
-      <c r="R11" s="20" t="n">
+      <c r="R11" s="21" t="n">
         <v>-0.1983</v>
       </c>
-      <c r="S11" s="13" t="n">
+      <c r="S11" s="14" t="n">
         <v>567535</v>
       </c>
-      <c r="T11" s="18" t="n">
+      <c r="T11" s="19" t="n">
         <v>1.73</v>
       </c>
-      <c r="U11" s="15" t="n">
+      <c r="U11" s="16" t="n">
         <v>1.29</v>
       </c>
-      <c r="V11" s="15" t="n">
+      <c r="V11" s="16" t="n">
         <v>2.35</v>
       </c>
-      <c r="W11" s="15" t="n">
+      <c r="W11" s="16" t="n">
         <v>0.44</v>
       </c>
-      <c r="X11" s="12" t="inlineStr"/>
-      <c r="Y11" s="13" t="n">
+      <c r="X11" s="13" t="inlineStr"/>
+      <c r="Y11" s="14" t="n">
         <v>22000</v>
       </c>
-      <c r="Z11" s="12" t="inlineStr">
+      <c r="Z11" s="13" t="inlineStr">
         <is>
           <t>⚠️余裕+0.80→+0.44に急落</t>
         </is>
       </c>
-      <c r="AA11" s="16" t="inlineStr">
+      <c r="AA11" s="17" t="inlineStr">
         <is>
           <t>①7/25に購入2件と急落、7日余裕+0.80→+0.44。悪化トレンド ②原価率22.4%は健全、広告費率57.7%が主因＝広告の問題 ③7/29判定。CR差し替えが本命、素材がなければ複製リセット ④消化率90%</t>
         </is>
@@ -2065,74 +2082,74 @@
           <t>ムダ毛シェーバー</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="6" t="n">
         <v>227240</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>106324</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="6" t="n">
         <v>90726</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="6" t="n">
         <v>30190</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="18" t="n">
         <v>0.1329</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="9" t="n">
         <v>0.4679</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="7" t="n">
         <v>0.3993</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="6" t="n">
         <v>83720</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="6" t="n">
         <v>39172</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="K12" s="6" t="n">
         <v>33860</v>
       </c>
-      <c r="L12" s="5" t="n">
+      <c r="L12" s="6" t="n">
         <v>10688</v>
       </c>
-      <c r="M12" s="17" t="n">
+      <c r="M12" s="18" t="n">
         <v>0.1277</v>
       </c>
-      <c r="N12" s="5" t="n">
+      <c r="N12" s="6" t="n">
         <v>35880</v>
       </c>
-      <c r="O12" s="5" t="n">
+      <c r="O12" s="6" t="n">
         <v>16788</v>
       </c>
-      <c r="P12" s="5" t="n">
+      <c r="P12" s="6" t="n">
         <v>11441</v>
       </c>
-      <c r="Q12" s="5" t="n">
+      <c r="Q12" s="6" t="n">
         <v>7651</v>
       </c>
-      <c r="R12" s="17" t="n">
+      <c r="R12" s="18" t="n">
         <v>0.2132</v>
       </c>
-      <c r="S12" s="5" t="n">
+      <c r="S12" s="6" t="n">
         <v>55759</v>
       </c>
-      <c r="T12" s="18" t="n">
+      <c r="T12" s="19" t="n">
         <v>2.5</v>
       </c>
-      <c r="U12" s="10" t="n">
+      <c r="U12" s="11" t="n">
         <v>1.88</v>
       </c>
-      <c r="V12" s="10" t="n">
+      <c r="V12" s="11" t="n">
         <v>5.49</v>
       </c>
-      <c r="W12" s="10" t="n">
+      <c r="W12" s="11" t="n">
         <v>0.62</v>
       </c>
       <c r="X12" s="4" t="inlineStr"/>
-      <c r="Y12" s="5" t="n">
+      <c r="Y12" s="6" t="n">
         <v>13000</v>
       </c>
       <c r="Z12" s="4" t="inlineStr">
@@ -2140,94 +2157,94 @@
           <t>✅黒字+30,190(7/27判定)</t>
         </is>
       </c>
-      <c r="AA12" s="11" t="inlineStr">
+      <c r="AA12" s="12" t="inlineStr">
         <is>
           <t>①7日利益+30,190に改善、余裕+0.63。7/27判定 ②原価率46.8%が最大の問題＝広告では直らない ③5,980→6,980円値上げは23.9%減まで許容＝値上げ最優先候補 ④CJ原価2,798円は交渉余地あり</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>接触冷感UVアームカバー</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="14" t="n">
         <v>226860</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>44688</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <v>118806</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <v>63366</v>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="18" t="n">
         <v>0.2793</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G13" s="15" t="n">
         <v>0.197</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="9" t="n">
         <v>0.5237000000000001</v>
       </c>
-      <c r="I13" s="13" t="n">
+      <c r="I13" s="14" t="n">
         <v>115420</v>
       </c>
-      <c r="J13" s="13" t="n">
+      <c r="J13" s="14" t="n">
         <v>22736</v>
       </c>
-      <c r="K13" s="13" t="n">
+      <c r="K13" s="14" t="n">
         <v>50067</v>
       </c>
-      <c r="L13" s="13" t="n">
+      <c r="L13" s="14" t="n">
         <v>42617</v>
       </c>
-      <c r="M13" s="14" t="n">
+      <c r="M13" s="15" t="n">
         <v>0.3692</v>
       </c>
-      <c r="N13" s="13" t="n">
+      <c r="N13" s="14" t="n">
         <v>47760</v>
       </c>
-      <c r="O13" s="13" t="n">
+      <c r="O13" s="14" t="n">
         <v>9408</v>
       </c>
-      <c r="P13" s="13" t="n">
+      <c r="P13" s="14" t="n">
         <v>16054</v>
       </c>
-      <c r="Q13" s="13" t="n">
+      <c r="Q13" s="14" t="n">
         <v>22298</v>
       </c>
-      <c r="R13" s="14" t="n">
+      <c r="R13" s="15" t="n">
         <v>0.4669</v>
       </c>
-      <c r="S13" s="13" t="n">
+      <c r="S13" s="14" t="n">
         <v>394568</v>
       </c>
-      <c r="T13" s="18" t="n">
+      <c r="T13" s="19" t="n">
         <v>1.91</v>
       </c>
-      <c r="U13" s="15" t="n">
+      <c r="U13" s="16" t="n">
         <v>1.25</v>
       </c>
-      <c r="V13" s="15" t="n">
+      <c r="V13" s="16" t="n">
         <v>2.21</v>
       </c>
-      <c r="W13" s="15" t="n">
+      <c r="W13" s="16" t="n">
         <v>0.66</v>
       </c>
-      <c r="X13" s="12" t="inlineStr"/>
-      <c r="Y13" s="13" t="n">
+      <c r="X13" s="13" t="inlineStr"/>
+      <c r="Y13" s="14" t="n">
         <v>17000</v>
       </c>
-      <c r="Z13" s="12" t="inlineStr">
+      <c r="Z13" s="13" t="inlineStr">
         <is>
           <t>👀7/29判定</t>
         </is>
       </c>
-      <c r="AA13" s="16" t="inlineStr">
+      <c r="AA13" s="17" t="inlineStr">
         <is>
           <t>①消化率98%天井だが余裕+0.66で増額ライン未達 ②原価率19.7%は極めて良い、広告費率52.4%が主因 ③売価3,980円でAOVが小さい→パーカー/UVハットとのセット販売が本命 ④7/29判定</t>
         </is>
@@ -2239,74 +2256,74 @@
           <t>瞬間冷感ポンチョ</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <v>206960</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>51324</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="6" t="n">
         <v>90504</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="6" t="n">
         <v>65132</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="7" t="n">
         <v>0.3147</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>0.248</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="9" t="n">
         <v>0.4373</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="6" t="n">
         <v>127360</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="6" t="n">
         <v>31584</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="K14" s="6" t="n">
         <v>37218</v>
       </c>
-      <c r="L14" s="5" t="n">
+      <c r="L14" s="6" t="n">
         <v>58558</v>
       </c>
-      <c r="M14" s="6" t="n">
+      <c r="M14" s="7" t="n">
         <v>0.4598</v>
       </c>
-      <c r="N14" s="5" t="n">
+      <c r="N14" s="6" t="n">
         <v>27860</v>
       </c>
-      <c r="O14" s="5" t="n">
+      <c r="O14" s="6" t="n">
         <v>6909</v>
       </c>
-      <c r="P14" s="5" t="n">
+      <c r="P14" s="6" t="n">
         <v>12949</v>
       </c>
-      <c r="Q14" s="5" t="n">
+      <c r="Q14" s="6" t="n">
         <v>8002</v>
       </c>
-      <c r="R14" s="17" t="n">
+      <c r="R14" s="18" t="n">
         <v>0.2872</v>
       </c>
-      <c r="S14" s="5" t="n">
+      <c r="S14" s="6" t="n">
         <v>133083</v>
       </c>
-      <c r="T14" s="18" t="n">
+      <c r="T14" s="19" t="n">
         <v>2.29</v>
       </c>
-      <c r="U14" s="10" t="n">
+      <c r="U14" s="11" t="n">
         <v>1.33</v>
       </c>
-      <c r="V14" s="10" t="n">
+      <c r="V14" s="11" t="n">
         <v>2.49</v>
       </c>
-      <c r="W14" s="10" t="n">
+      <c r="W14" s="11" t="n">
         <v>0.96</v>
       </c>
       <c r="X14" s="4" t="inlineStr"/>
-      <c r="Y14" s="5" t="n">
+      <c r="Y14" s="6" t="n">
         <v>13000</v>
       </c>
       <c r="Z14" s="4" t="inlineStr">
@@ -2314,94 +2331,94 @@
           <t>✅余裕+0.96に改善</t>
         </is>
       </c>
-      <c r="AA14" s="11" t="inlineStr">
+      <c r="AA14" s="12" t="inlineStr">
         <is>
           <t>①余裕+0.40→+0.96に改善、利益率31.5% ②消化率95%天井 ③原価率24.8%は良好 ④夏物で最も季節性が強い。8月中旬から縮小</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>健康サンダル</t>
         </is>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="14" t="n">
         <v>179280</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>39508</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <v>90907</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <v>48865</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="18" t="n">
         <v>0.2726</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G15" s="15" t="n">
         <v>0.2204</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="9" t="n">
         <v>0.5071</v>
       </c>
-      <c r="I15" s="13" t="n">
+      <c r="I15" s="14" t="n">
         <v>84660</v>
       </c>
-      <c r="J15" s="13" t="n">
+      <c r="J15" s="14" t="n">
         <v>17430</v>
       </c>
-      <c r="K15" s="13" t="n">
+      <c r="K15" s="14" t="n">
         <v>39935</v>
       </c>
-      <c r="L15" s="13" t="n">
+      <c r="L15" s="14" t="n">
         <v>27295</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="M15" s="15" t="n">
         <v>0.3224</v>
       </c>
-      <c r="N15" s="13" t="n">
+      <c r="N15" s="14" t="n">
         <v>19920</v>
       </c>
-      <c r="O15" s="13" t="n">
+      <c r="O15" s="14" t="n">
         <v>4648</v>
       </c>
-      <c r="P15" s="13" t="n">
+      <c r="P15" s="14" t="n">
         <v>13335</v>
       </c>
-      <c r="Q15" s="13" t="n">
+      <c r="Q15" s="14" t="n">
         <v>1937</v>
       </c>
-      <c r="R15" s="17" t="n">
+      <c r="R15" s="18" t="n">
         <v>0.09719999999999999</v>
       </c>
-      <c r="S15" s="13" t="n">
+      <c r="S15" s="14" t="n">
         <v>320815</v>
       </c>
-      <c r="T15" s="18" t="n">
+      <c r="T15" s="19" t="n">
         <v>1.97</v>
       </c>
-      <c r="U15" s="15" t="n">
+      <c r="U15" s="16" t="n">
         <v>1.28</v>
       </c>
-      <c r="V15" s="15" t="n">
+      <c r="V15" s="16" t="n">
         <v>2.33</v>
       </c>
-      <c r="W15" s="15" t="n">
+      <c r="W15" s="16" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="X15" s="12" t="inlineStr"/>
-      <c r="Y15" s="13" t="n">
+      <c r="X15" s="13" t="inlineStr"/>
+      <c r="Y15" s="14" t="n">
         <v>13000</v>
       </c>
-      <c r="Z15" s="12" t="inlineStr">
+      <c r="Z15" s="13" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="AA15" s="16" t="inlineStr">
+      <c r="AA15" s="17" t="inlineStr">
         <is>
           <t>①消化率102%天井、余裕+0.69 ②原価率22.0%は良好、広告費率50.7%が主因 ③18サイズ展開でサイズ選択UIの改善がCVR向上の本命 ④秋以降も需要継続する非季節商品</t>
         </is>
@@ -2413,74 +2430,74 @@
           <t>携帯電動シェーバー</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="6" t="n">
         <v>159360</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="6" t="n">
         <v>54033</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="6" t="n">
         <v>76795</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="6" t="n">
         <v>28532</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="18" t="n">
         <v>0.179</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="9" t="n">
         <v>0.3391</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="9" t="n">
         <v>0.4819</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="6" t="n">
         <v>39840</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="6" t="n">
         <v>13944</v>
       </c>
-      <c r="K16" s="5" t="n">
+      <c r="K16" s="6" t="n">
         <v>30945</v>
       </c>
-      <c r="L16" s="19" t="n">
+      <c r="L16" s="20" t="n">
         <v>-5049</v>
       </c>
-      <c r="M16" s="20" t="n">
+      <c r="M16" s="21" t="n">
         <v>-0.1267</v>
       </c>
-      <c r="N16" s="5" t="n">
+      <c r="N16" s="6" t="n">
         <v>19920</v>
       </c>
-      <c r="O16" s="5" t="n">
+      <c r="O16" s="6" t="n">
         <v>6972</v>
       </c>
-      <c r="P16" s="5" t="n">
+      <c r="P16" s="6" t="n">
         <v>10085</v>
       </c>
-      <c r="Q16" s="5" t="n">
+      <c r="Q16" s="6" t="n">
         <v>2863</v>
       </c>
-      <c r="R16" s="17" t="n">
+      <c r="R16" s="18" t="n">
         <v>0.1437</v>
       </c>
-      <c r="S16" s="5" t="n">
+      <c r="S16" s="6" t="n">
         <v>207251</v>
       </c>
-      <c r="T16" s="18" t="n">
+      <c r="T16" s="19" t="n">
         <v>2.08</v>
       </c>
-      <c r="U16" s="10" t="n">
+      <c r="U16" s="11" t="n">
         <v>1.51</v>
       </c>
-      <c r="V16" s="10" t="n">
+      <c r="V16" s="11" t="n">
         <v>3.22</v>
       </c>
-      <c r="W16" s="10" t="n">
+      <c r="W16" s="11" t="n">
         <v>0.57</v>
       </c>
       <c r="X16" s="4" t="inlineStr"/>
-      <c r="Y16" s="5" t="n">
+      <c r="Y16" s="6" t="n">
         <v>11000</v>
       </c>
       <c r="Z16" s="4" t="inlineStr">
@@ -2488,94 +2505,94 @@
           <t>👀8/1判定</t>
         </is>
       </c>
-      <c r="AA16" s="11" t="inlineStr">
+      <c r="AA16" s="12" t="inlineStr">
         <is>
           <t>①余裕+0.33→+0.56に改善、7日利益+28,532 ②日販4.4個でブレ±64pt＝利益率では判断不能、7日累計で見る ③8/1判定 ④原価率33.9%・広告費率48.2%の両方が重い</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>UV歯ブラシ除菌器</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="14" t="n">
         <v>134700</v>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="14" t="n">
         <v>48600</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="14" t="n">
         <v>80486</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="14" t="n">
         <v>5614</v>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="18" t="n">
         <v>0.0417</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="9" t="n">
         <v>0.3608</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="9" t="n">
         <v>0.5975</v>
       </c>
-      <c r="I17" s="13" t="n">
+      <c r="I17" s="14" t="n">
         <v>80820</v>
       </c>
-      <c r="J17" s="13" t="n">
+      <c r="J17" s="14" t="n">
         <v>29160</v>
       </c>
-      <c r="K17" s="13" t="n">
+      <c r="K17" s="14" t="n">
         <v>29670</v>
       </c>
-      <c r="L17" s="13" t="n">
+      <c r="L17" s="14" t="n">
         <v>21990</v>
       </c>
-      <c r="M17" s="17" t="n">
+      <c r="M17" s="18" t="n">
         <v>0.2721</v>
       </c>
-      <c r="N17" s="13" t="n">
+      <c r="N17" s="14" t="n">
         <v>35920</v>
       </c>
-      <c r="O17" s="13" t="n">
+      <c r="O17" s="14" t="n">
         <v>12960</v>
       </c>
-      <c r="P17" s="13" t="n">
+      <c r="P17" s="14" t="n">
         <v>8224</v>
       </c>
-      <c r="Q17" s="13" t="n">
+      <c r="Q17" s="14" t="n">
         <v>14736</v>
       </c>
-      <c r="R17" s="14" t="n">
+      <c r="R17" s="15" t="n">
         <v>0.4102</v>
       </c>
-      <c r="S17" s="13" t="n">
+      <c r="S17" s="14" t="n">
         <v>270885</v>
       </c>
-      <c r="T17" s="18" t="n">
+      <c r="T17" s="19" t="n">
         <v>1.67</v>
       </c>
-      <c r="U17" s="15" t="n">
+      <c r="U17" s="16" t="n">
         <v>1.56</v>
       </c>
-      <c r="V17" s="15" t="n">
+      <c r="V17" s="16" t="n">
         <v>3.46</v>
       </c>
-      <c r="W17" s="15" t="n">
+      <c r="W17" s="16" t="n">
         <v>0.11</v>
       </c>
-      <c r="X17" s="12" t="inlineStr"/>
-      <c r="Y17" s="13" t="n">
+      <c r="X17" s="13" t="inlineStr"/>
+      <c r="Y17" s="14" t="n">
         <v>10000</v>
       </c>
-      <c r="Z17" s="12" t="inlineStr">
+      <c r="Z17" s="13" t="inlineStr">
         <is>
           <t>🔧黒字転換+5,614(7/30判定)</t>
         </is>
       </c>
-      <c r="AA17" s="16" t="inlineStr">
+      <c r="AA17" s="17" t="inlineStr">
         <is>
           <t>①7日利益 -5,129→+5,614に黒字転換＝複製リセットが効いた ②広告費率59.8%はまだ重い ③7/30判定。余裕+0.11と薄いので改善継続が条件 ④売価8,980円で値上げ余地は小さい(8.0%減まで)</t>
         </is>
@@ -2587,74 +2604,74 @@
           <t>壁掛けディスペンサー</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="6" t="n">
         <v>100700</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="6" t="n">
         <v>35732</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="6" t="n">
         <v>87075</v>
       </c>
-      <c r="E18" s="19" t="n">
+      <c r="E18" s="20" t="n">
         <v>-22107</v>
       </c>
-      <c r="F18" s="20" t="n">
+      <c r="F18" s="21" t="n">
         <v>-0.2195</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="9" t="n">
         <v>0.3548</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="9" t="n">
         <v>0.8647</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="6" t="n">
         <v>45860</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="6" t="n">
         <v>16055</v>
       </c>
-      <c r="K18" s="5" t="n">
+      <c r="K18" s="6" t="n">
         <v>34494</v>
       </c>
-      <c r="L18" s="19" t="n">
+      <c r="L18" s="20" t="n">
         <v>-4689</v>
       </c>
-      <c r="M18" s="20" t="n">
+      <c r="M18" s="21" t="n">
         <v>-0.1022</v>
       </c>
-      <c r="N18" s="5" t="n">
+      <c r="N18" s="6" t="n">
         <v>13960</v>
       </c>
-      <c r="O18" s="5" t="n">
+      <c r="O18" s="6" t="n">
         <v>5056</v>
       </c>
-      <c r="P18" s="5" t="n">
+      <c r="P18" s="6" t="n">
         <v>11000</v>
       </c>
-      <c r="Q18" s="19" t="n">
+      <c r="Q18" s="20" t="n">
         <v>-2096</v>
       </c>
-      <c r="R18" s="20" t="n">
+      <c r="R18" s="21" t="n">
         <v>-0.1501</v>
       </c>
-      <c r="S18" s="5" t="n">
+      <c r="S18" s="6" t="n">
         <v>103812</v>
       </c>
-      <c r="T18" s="18" t="n">
+      <c r="T18" s="19" t="n">
         <v>1.16</v>
       </c>
-      <c r="U18" s="10" t="n">
+      <c r="U18" s="11" t="n">
         <v>1.55</v>
       </c>
-      <c r="V18" s="10" t="n">
+      <c r="V18" s="11" t="n">
         <v>3.39</v>
       </c>
-      <c r="W18" s="10" t="n">
+      <c r="W18" s="11" t="n">
         <v>-0.39</v>
       </c>
       <c r="X18" s="4" t="inlineStr"/>
-      <c r="Y18" s="5" t="n">
+      <c r="Y18" s="6" t="n">
         <v>6000</v>
       </c>
       <c r="Z18" s="4" t="inlineStr">
@@ -2662,92 +2679,92 @@
           <t>🚨6kに半減済(8/1早期判定)</t>
         </is>
       </c>
-      <c r="AA18" s="11" t="inlineStr">
+      <c r="AA18" s="12" t="inlineStr">
         <is>
           <t>①類似5%停止で6kに半減済。7/25消化11,000円は停止前の残り ②広告費率86.5%＝構造的に成立していない ③8/1にCPA&gt;6,000なら早期停止、8/6最終判定 ④週50CVに必要な44,887円/日は出せない</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>湯上がりガーゼワンピース</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="14" t="n">
         <v>80720</v>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="14" t="n">
         <v>27552</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="14" t="n">
         <v>48535</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="14" t="n">
         <v>4633</v>
       </c>
-      <c r="F19" s="17" t="n">
+      <c r="F19" s="18" t="n">
         <v>0.0574</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="9" t="n">
         <v>0.3413</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="9" t="n">
         <v>0.6012999999999999</v>
       </c>
-      <c r="I19" s="13" t="n">
+      <c r="I19" s="14" t="n">
         <v>5980</v>
       </c>
-      <c r="J19" s="13" t="n">
+      <c r="J19" s="14" t="n">
         <v>1968</v>
       </c>
-      <c r="K19" s="13" t="n">
+      <c r="K19" s="14" t="n">
         <v>17833</v>
       </c>
-      <c r="L19" s="21" t="n">
+      <c r="L19" s="22" t="n">
         <v>-13821</v>
       </c>
-      <c r="M19" s="20" t="n">
+      <c r="M19" s="21" t="n">
         <v>-2.3112</v>
       </c>
-      <c r="N19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="13" t="n">
+      <c r="N19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="14" t="n">
         <v>5379</v>
       </c>
-      <c r="Q19" s="21" t="n">
+      <c r="Q19" s="22" t="n">
         <v>-5379</v>
       </c>
-      <c r="R19" s="12" t="inlineStr"/>
-      <c r="S19" s="13" t="n">
+      <c r="R19" s="13" t="inlineStr"/>
+      <c r="S19" s="14" t="n">
         <v>106500</v>
       </c>
-      <c r="T19" s="18" t="n">
+      <c r="T19" s="19" t="n">
         <v>1.66</v>
       </c>
-      <c r="U19" s="15" t="n">
+      <c r="U19" s="16" t="n">
         <v>1.52</v>
       </c>
-      <c r="V19" s="15" t="n">
+      <c r="V19" s="16" t="n">
         <v>3.24</v>
       </c>
-      <c r="W19" s="15" t="n">
+      <c r="W19" s="16" t="n">
         <v>0.14</v>
       </c>
-      <c r="X19" s="12" t="inlineStr"/>
-      <c r="Y19" s="13" t="n">
+      <c r="X19" s="13" t="inlineStr"/>
+      <c r="Y19" s="14" t="n">
         <v>6500</v>
       </c>
-      <c r="Z19" s="12" t="inlineStr">
+      <c r="Z19" s="13" t="inlineStr">
         <is>
           <t>🚨判定不合格(余裕+0.14&lt;+0.30)</t>
         </is>
       </c>
-      <c r="AA19" s="16" t="inlineStr">
+      <c r="AA19" s="17" t="inlineStr">
         <is>
           <t>①★7/26判定で不合格（余裕+0.14 &lt; 基準+0.30）→停止 ②黒字転換はしたが日次利益662円と僅少、広告費率60.1% ③6,500円/日を4WAY(増分MER3.34)に回すと+7,668円/日＝11倍 ④夏物で9月以降の価値は低い</t>
         </is>
@@ -2759,74 +2776,74 @@
           <t>バランスケアスリッパ</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="6" t="n">
         <v>79680</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="6" t="n">
         <v>20864</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="6" t="n">
         <v>52332</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="6" t="n">
         <v>6484</v>
       </c>
-      <c r="F20" s="17" t="n">
+      <c r="F20" s="18" t="n">
         <v>0.0814</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="7" t="n">
         <v>0.2618</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="9" t="n">
         <v>0.6568000000000001</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="6" t="n">
         <v>19920</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="J20" s="6" t="n">
         <v>5216</v>
       </c>
-      <c r="K20" s="5" t="n">
+      <c r="K20" s="6" t="n">
         <v>14589</v>
       </c>
-      <c r="L20" s="5" t="n">
+      <c r="L20" s="6" t="n">
         <v>115</v>
       </c>
-      <c r="M20" s="17" t="n">
+      <c r="M20" s="18" t="n">
         <v>0.0058</v>
       </c>
-      <c r="N20" s="5" t="n">
+      <c r="N20" s="6" t="n">
         <v>14940</v>
       </c>
-      <c r="O20" s="5" t="n">
+      <c r="O20" s="6" t="n">
         <v>3912</v>
       </c>
-      <c r="P20" s="5" t="n">
+      <c r="P20" s="6" t="n">
         <v>4117</v>
       </c>
-      <c r="Q20" s="5" t="n">
+      <c r="Q20" s="6" t="n">
         <v>6911</v>
       </c>
-      <c r="R20" s="6" t="n">
+      <c r="R20" s="7" t="n">
         <v>0.4626</v>
       </c>
-      <c r="S20" s="5" t="n">
+      <c r="S20" s="6" t="n">
         <v>96139</v>
       </c>
-      <c r="T20" s="18" t="n">
+      <c r="T20" s="19" t="n">
         <v>1.52</v>
       </c>
-      <c r="U20" s="10" t="n">
+      <c r="U20" s="11" t="n">
         <v>1.35</v>
       </c>
-      <c r="V20" s="10" t="n">
+      <c r="V20" s="11" t="n">
         <v>2.58</v>
       </c>
-      <c r="W20" s="10" t="n">
+      <c r="W20" s="11" t="n">
         <v>0.17</v>
       </c>
       <c r="X20" s="4" t="inlineStr"/>
-      <c r="Y20" s="5" t="n">
+      <c r="Y20" s="6" t="n">
         <v>5000</v>
       </c>
       <c r="Z20" s="4" t="inlineStr">
@@ -2834,84 +2851,84 @@
           <t>🔧黒字+6,484(7/29判定)</t>
         </is>
       </c>
-      <c r="AA20" s="11" t="inlineStr">
+      <c r="AA20" s="12" t="inlineStr">
         <is>
           <t>①7日利益+6,484、余裕+0.17 ②広告費率65.7%が主因、原価率26.2%は良好 ③増分MER0.00＝減らしても売上が落ちない。7/29判定で5k→3kも選択肢 ④非季節商品</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>瞬間冷却ハンディファン</t>
         </is>
       </c>
-      <c r="B21" s="13" t="n">
+      <c r="B21" s="14" t="n">
         <v>41860</v>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="14" t="n">
         <v>14371</v>
       </c>
-      <c r="D21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="13" t="n">
+      <c r="D21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="14" t="n">
         <v>27489</v>
       </c>
-      <c r="F21" s="14" t="n">
+      <c r="F21" s="15" t="n">
         <v>0.6567</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="9" t="n">
         <v>0.3433</v>
       </c>
-      <c r="H21" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="13" t="n">
+      <c r="H21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="14" t="n">
         <v>11960</v>
       </c>
-      <c r="J21" s="13" t="n">
+      <c r="J21" s="14" t="n">
         <v>4106</v>
       </c>
-      <c r="K21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="13" t="n">
+      <c r="K21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="14" t="n">
         <v>7854</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="M21" s="15" t="n">
         <v>0.6567</v>
       </c>
-      <c r="N21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="12" t="inlineStr"/>
-      <c r="S21" s="13" t="n">
+      <c r="N21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="13" t="inlineStr"/>
+      <c r="S21" s="14" t="n">
         <v>70686</v>
       </c>
-      <c r="T21" s="12" t="inlineStr"/>
-      <c r="U21" s="12" t="inlineStr"/>
-      <c r="V21" s="15" t="n">
+      <c r="T21" s="13" t="inlineStr"/>
+      <c r="U21" s="13" t="inlineStr"/>
+      <c r="V21" s="16" t="n">
         <v>3.26</v>
       </c>
-      <c r="W21" s="12" t="inlineStr"/>
-      <c r="X21" s="12" t="inlineStr"/>
-      <c r="Y21" s="12" t="inlineStr"/>
-      <c r="Z21" s="12" t="inlineStr">
+      <c r="W21" s="13" t="inlineStr"/>
+      <c r="X21" s="13" t="inlineStr"/>
+      <c r="Y21" s="13" t="inlineStr"/>
+      <c r="Z21" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA21" s="16" t="inlineStr">
+      <c r="AA21" s="17" t="inlineStr">
         <is>
           <t>①広告ゼロで7日利益+33,264。4WAYからの流入 ②広告は出さない（4WAYと共食い） ③在庫消化用として現状維持</t>
         </is>
@@ -2923,63 +2940,63 @@
           <t>優先配送</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B22" s="6" t="n">
         <v>40200</v>
       </c>
-      <c r="C22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5" t="n">
+      <c r="C22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6" t="n">
         <v>40200</v>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F22" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="5" t="n">
+      <c r="G22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6" t="n">
         <v>15544</v>
       </c>
-      <c r="J22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="5" t="n">
+      <c r="J22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6" t="n">
         <v>15544</v>
       </c>
-      <c r="M22" s="6" t="n">
+      <c r="M22" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="N22" s="5" t="n">
+      <c r="N22" s="6" t="n">
         <v>3216</v>
       </c>
-      <c r="O22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="5" t="n">
+      <c r="O22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="6" t="n">
         <v>3216</v>
       </c>
-      <c r="R22" s="6" t="n">
+      <c r="R22" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="S22" s="5" t="n">
+      <c r="S22" s="6" t="n">
         <v>113632</v>
       </c>
       <c r="T22" s="4" t="inlineStr"/>
       <c r="U22" s="4" t="inlineStr"/>
-      <c r="V22" s="10" t="n">
+      <c r="V22" s="11" t="n">
         <v>1.54</v>
       </c>
       <c r="W22" s="4" t="inlineStr"/>
@@ -2990,84 +3007,84 @@
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA22" s="11" t="inlineStr">
+      <c r="AA22" s="12" t="inlineStr">
         <is>
           <t>①7日75件/1,713注文＝アタッチ率4.38%（前週3.49%から改善） ②原価0＝売上全額が利益 ③15%到達で+141,156円/7日・利益率+0.94pt ④低単価帯(〜3,980円)のアタッチ率0%が最大の伸びしろ</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>完全遮光・接触冷感UVハット</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="14" t="n">
         <v>11960</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="14" t="n">
         <v>2822</v>
       </c>
-      <c r="D23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="13" t="n">
+      <c r="D23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="14" t="n">
         <v>9138</v>
       </c>
-      <c r="F23" s="14" t="n">
+      <c r="F23" s="15" t="n">
         <v>0.764</v>
       </c>
-      <c r="G23" s="14" t="n">
+      <c r="G23" s="15" t="n">
         <v>0.236</v>
       </c>
-      <c r="H23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="13" t="n">
+      <c r="H23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="14" t="n">
         <v>5980</v>
       </c>
-      <c r="J23" s="13" t="n">
+      <c r="J23" s="14" t="n">
         <v>1411</v>
       </c>
-      <c r="K23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="13" t="n">
+      <c r="K23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="14" t="n">
         <v>4569</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="M23" s="15" t="n">
         <v>0.764</v>
       </c>
-      <c r="N23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="12" t="inlineStr"/>
-      <c r="S23" s="13" t="n">
+      <c r="N23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="13" t="inlineStr"/>
+      <c r="S23" s="14" t="n">
         <v>41121</v>
       </c>
-      <c r="T23" s="12" t="inlineStr"/>
-      <c r="U23" s="12" t="inlineStr"/>
-      <c r="V23" s="15" t="n">
+      <c r="T23" s="13" t="inlineStr"/>
+      <c r="U23" s="13" t="inlineStr"/>
+      <c r="V23" s="16" t="n">
         <v>2.42</v>
       </c>
-      <c r="W23" s="12" t="inlineStr"/>
-      <c r="X23" s="12" t="inlineStr"/>
-      <c r="Y23" s="12" t="inlineStr"/>
-      <c r="Z23" s="12" t="inlineStr">
+      <c r="W23" s="13" t="inlineStr"/>
+      <c r="X23" s="13" t="inlineStr"/>
+      <c r="Y23" s="13" t="inlineStr"/>
+      <c r="Z23" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA23" s="16" t="inlineStr">
+      <c r="AA23" s="17" t="inlineStr">
         <is>
           <t>①広告ゼロ・利益率76.4% ②日傘/パーカーとのセット販売でクロスセルが本命 ③秋の帽子需要期(10月)に単独テスト候補</t>
         </is>
@@ -3079,59 +3096,59 @@
           <t>リカバリーサンダル</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B24" s="6" t="n">
         <v>3980</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="6" t="n">
         <v>1309</v>
       </c>
-      <c r="D24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="5" t="n">
+      <c r="D24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="6" t="n">
         <v>2671</v>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F24" s="7" t="n">
         <v>0.6711</v>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G24" s="7" t="n">
         <v>0.3289</v>
       </c>
-      <c r="H24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="5" t="n">
+      <c r="H24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="5" t="n">
+      <c r="N24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R24" s="4" t="inlineStr"/>
-      <c r="S24" s="5" t="n">
+      <c r="S24" s="6" t="n">
         <v>18697</v>
       </c>
       <c r="T24" s="4" t="inlineStr"/>
       <c r="U24" s="4" t="inlineStr"/>
-      <c r="V24" s="10" t="n">
+      <c r="V24" s="11" t="n">
         <v>3.11</v>
       </c>
       <c r="W24" s="4" t="inlineStr"/>
@@ -3142,74 +3159,74 @@
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA24" s="11" t="inlineStr">
+      <c r="AA24" s="12" t="inlineStr">
         <is>
           <t>①30日7個。8月で需要終了、今から出稿する価値なし ②来春(4月)のテスト枠候補</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>ネックマッサージャー</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="12" t="inlineStr"/>
-      <c r="G25" s="12" t="inlineStr"/>
-      <c r="H25" s="12" t="inlineStr"/>
-      <c r="I25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="12" t="inlineStr"/>
-      <c r="N25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="12" t="inlineStr"/>
-      <c r="S25" s="13" t="n">
+      <c r="B25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="13" t="inlineStr"/>
+      <c r="G25" s="13" t="inlineStr"/>
+      <c r="H25" s="13" t="inlineStr"/>
+      <c r="I25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="13" t="inlineStr"/>
+      <c r="N25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="13" t="inlineStr"/>
+      <c r="S25" s="14" t="n">
         <v>6946</v>
       </c>
-      <c r="T25" s="12" t="inlineStr"/>
-      <c r="U25" s="12" t="inlineStr"/>
-      <c r="V25" s="12" t="inlineStr"/>
-      <c r="W25" s="12" t="inlineStr"/>
-      <c r="X25" s="12" t="inlineStr"/>
-      <c r="Y25" s="12" t="inlineStr"/>
-      <c r="Z25" s="12" t="inlineStr">
+      <c r="T25" s="13" t="inlineStr"/>
+      <c r="U25" s="13" t="inlineStr"/>
+      <c r="V25" s="13" t="inlineStr"/>
+      <c r="W25" s="13" t="inlineStr"/>
+      <c r="X25" s="13" t="inlineStr"/>
+      <c r="Y25" s="13" t="inlineStr"/>
+      <c r="Z25" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA25" s="16" t="inlineStr">
+      <c r="AA25" s="17" t="inlineStr">
         <is>
           <t>①30日1個。売価9,980円・原価率30.4%は良好 ②秋冬需要（肩こり・ギフト）→11月テスト枠候補 ③今は何もしない</t>
         </is>
@@ -3221,48 +3238,48 @@
           <t>姿勢サポートベルト</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="5" t="n">
+      <c r="B26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="4" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="5" t="n">
+      <c r="I26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="5" t="n">
+      <c r="N26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R26" s="4" t="inlineStr"/>
-      <c r="S26" s="5" t="n">
+      <c r="S26" s="6" t="n">
         <v>4551</v>
       </c>
       <c r="T26" s="4" t="inlineStr"/>
@@ -3276,74 +3293,74 @@
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA26" s="11" t="inlineStr">
+      <c r="AA26" s="12" t="inlineStr">
         <is>
           <t>①30日1個。原価率24.1%は良好だが需要が立っていない ②在庫リスクなし、放置で可</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>癒しの指圧マット</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="12" t="inlineStr"/>
-      <c r="G27" s="12" t="inlineStr"/>
-      <c r="H27" s="12" t="inlineStr"/>
-      <c r="I27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="12" t="inlineStr"/>
-      <c r="N27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="12" t="inlineStr"/>
-      <c r="S27" s="13" t="n">
+      <c r="B27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr"/>
+      <c r="G27" s="13" t="inlineStr"/>
+      <c r="H27" s="13" t="inlineStr"/>
+      <c r="I27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="13" t="inlineStr"/>
+      <c r="N27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="13" t="inlineStr"/>
+      <c r="S27" s="14" t="n">
         <v>4332</v>
       </c>
-      <c r="T27" s="12" t="inlineStr"/>
-      <c r="U27" s="12" t="inlineStr"/>
-      <c r="V27" s="12" t="inlineStr"/>
-      <c r="W27" s="12" t="inlineStr"/>
-      <c r="X27" s="12" t="inlineStr"/>
-      <c r="Y27" s="12" t="inlineStr"/>
-      <c r="Z27" s="12" t="inlineStr">
+      <c r="T27" s="13" t="inlineStr"/>
+      <c r="U27" s="13" t="inlineStr"/>
+      <c r="V27" s="13" t="inlineStr"/>
+      <c r="W27" s="13" t="inlineStr"/>
+      <c r="X27" s="13" t="inlineStr"/>
+      <c r="Y27" s="13" t="inlineStr"/>
+      <c r="Z27" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA27" s="16" t="inlineStr">
+      <c r="AA27" s="17" t="inlineStr">
         <is>
           <t>①7/25改定で原価-262円と最大の値下げ、原価率27.6% ②秋冬の「おうち時間」需要でテスト枠候補</t>
         </is>
@@ -3355,48 +3372,48 @@
           <t>ナノバブルシャワーヘッド</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="5" t="n">
+      <c r="B28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="5" t="n">
+      <c r="I28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="5" t="n">
+      <c r="N28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R28" s="4" t="inlineStr"/>
-      <c r="S28" s="5" t="n">
+      <c r="S28" s="6" t="n">
         <v>51975</v>
       </c>
       <c r="T28" s="4" t="inlineStr"/>
@@ -3410,7 +3427,7 @@
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="AA28" s="11" t="inlineStr">
+      <c r="AA28" s="12" t="inlineStr">
         <is>
           <t>①30日7.7万円・広告ゼロ。原価率32.3%・分岐MER1.48 ②秋冬に需要増（入浴時間の増加） ③9月のテスト枠の第一候補</t>
         </is>

</xml_diff>

<commit_message>
Implement the decision flow and trace it in the workbook
Explaining the budget logic in prose let it drift from what I actually
recommended: today's ワンピース stop came from a criterion declared before
the reduction threshold moved to 余裕 < 0, and the written flow would have
said hold.

- Add scripts/decision_flow.py; judgments are now generated by judge()
  rather than written by hand
- New "判定フロー" sheet carries the flow (S-1..S5, C1..C2, V1..V4) and a
  per-product trace showing the branches taken and the budget delta
- Add S-1 (act only on a product's judgment day) and S2b (stop a
  profitable product when its budget earns more redeployed to a
  ceiling-bound, above-target product) — S2b is what actually justifies
  stopping ワンピース: 4,112 JPY/day redeployed against 662 JPY/day now

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-26.xlsx
+++ b/data/reports/report-2026-07-26.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="全体サマリー" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="商品別" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="判定フロー" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +60,35 @@
       <color rgb="00CC0000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +120,11 @@
         <fgColor rgb="00D6EFD8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1FB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -118,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +184,29 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -532,7 +589,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・7日/3日/前日を並列表示）</t>
+          <t>LOOTY 日次損益レポート 2026-07-26(日) 定例（昨日=7/25 土実績・判定フローシート追加）</t>
         </is>
       </c>
     </row>
@@ -959,68 +1016,75 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>・★判断軸がMERである理由: ①利益率=1−原価率−1/MER で数式が直結する ②商品別のMeta計上は突合率79〜108%とブレる（4WAY79%・サンダル79%・スリッパ108%）③Metaの数値は媒体の自己申告 ④カタログ広告など商品配賦できない費用も分母に入り帳尻が合う</t>
+          <t>・★シート「判定フロー」を追加。商品別シートの判定は、このフローを実装した関数から機械的に生成しており、フロー図と実際の判定が食い違わないようにしている。全商品がどの分岐を通ったかを追える</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>・★MERは「正確なROAS」ではなく別物。ROAS=Meta計上値(推定)÷広告費、MER=Shopify実売上(実測)÷広告費。MERは非広告流入も分子に含むため広告の貢献を過大評価する（7日実測でMetaは全店売上の96%を計上、非広告分は約4%=385,277円）。この弱点を埋めるのが増分MERで、MER=継続/停止の判定、増分MER=予算増減の判定と使い分ける</t>
+          <t>・★判断軸がMERである理由: ①利益率=1−原価率−1/MER で数式が直結する ②商品別のMeta計上は突合率79〜108%とブレる（4WAY79%・サンダル79%・スリッパ108%）③Metaの数値は媒体の自己申告 ④カタログ広告など商品配賦できない費用も分母に入り帳尻が合う</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>・★列を「7日 → 3日 → 前日」の順に並べ替え、3日も売上/原価/広告費/利益/利益率の5項目に拡張（前日も同じ5項目に統一）</t>
+          <t>・★MERは「正確なROAS」ではなく別物。ROAS=Meta計上値(推定)÷広告費、MER=Shopify実売上(実測)÷広告費。MERは非広告流入も分子に含むため広告の貢献を過大評価する（7日実測でMetaは全店売上の96%を計上、非広告分は約4%=385,277円）。この弱点を埋めるのが増分MERで、MER=継続/停止の判定、増分MER=予算増減の判定と使い分ける</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>・★目標MER列を追加。目標MER = 1 ÷ (1 − その商品の原価率 − 0.35)。商品ごとに2.17〜5.49と差が大きいため全店値2.91は使わない。MER列は目標超え=緑・未達=赤</t>
+          <t>・★列を「7日 → 3日 → 前日」の順に並べ替え、3日も売上/原価/広告費/利益/利益率の5項目に拡張（前日も同じ5項目に統一）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>・★3日利益率は全商品に表示（従来は日販20個以上に限定）。ただし日販10個未満の商品は日次のブレが13〜64ptあり、3日平均でも実力を測れない点は変わらない</t>
+          <t>・★目標MER列を追加。目標MER = 1 ÷ (1 − その商品の原価率 − 0.35)。商品ごとに2.17〜5.49と差が大きいため全店値2.91は使わない。MER列は目標超え=緑・未達=赤</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>・★7/26判定: 湯上がりガーゼワンピースは7日余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
+          <t>・★3日利益率は全商品に表示（従来は日販20個以上に限定）。ただし日販10個未満の商品は日次のブレが13〜64ptあり、3日平均でも実力を測れない点は変わらない</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>・★増額候補（自分の目標MER超え×消化率95%以上）: 害虫ブロッカー(2.78&gt;2.31・102%)・ナノガラス脱毛パッド(2.39&gt;2.17・100%)・完全遮光(2.70&gt;2.56・95%)</t>
+          <t>・★7/26判定: 湯上がりガーゼワンピースは7日余裕+0.14で合格基準+0.30に未達 → 停止（6,500円/日）</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>・全期間の広告費・原価はMeta/Shopifyの実測。推計・外挿は不使用</t>
+          <t>・★増額候補（自分の目標MER超え×消化率95%以上）: 害虫ブロッカー(2.78&gt;2.31・102%)・ナノガラス脱毛パッド(2.39&gt;2.17・100%)・完全遮光(2.70&gt;2.56・95%)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>・30日窓の途中開始: 卓上冷感クーラー7/13(13日)・5WAY腰掛けファン7/19(7日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10(16日)</t>
+          <t>・全期間の広告費・原価はMeta/Shopifyの実測。推計・外挿は不使用</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>・30日窓の途中開始: 卓上冷感クーラー7/13(13日)・5WAY腰掛けファン7/19(7日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10(16日)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>・増分MER: 7/22以降に予算を3,000円/日以上動かした商品がないため全商品「判定保留」</t>
         </is>
@@ -3436,4 +3500,1425 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="78" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>予算増減・CR投入の判定フロー　※商品別シートの判定はこのフローから機械的に生成している</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>【予算フロー】上から順に判定する</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>S-1</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>今日が この商品の判定日 か？</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>NO→据置（監視のみ）。判定日以外に予算を触らない ／ YES→S0へ　※例外: 事故（購入ゼロで分岐CPA×3を消化・CPM2倍）は即日対応</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>S0</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>日販10個未満か？</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>YES→利益率では判断しない。7日累計の金額とMERだけで判断する（日次のブレが13〜64ptあるため）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>7日利益 &gt; 0 か？</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>NO→撤退プロトコル(S1a)へ ／ YES→S2へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>S1a</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>日次赤字 ÷ 予算 ≥ 15%、またはテコ入れ2巡目か？</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>YES→予算半減＋テコ入れ ／ NO→予算据置＋CR追加し7日後に判定</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>MER ≥ その商品の目標MER か？</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>目標MER = 1÷(1−原価率−0.35)。商品ごとに2.17〜5.49と差が大きい。NO→S2aへ ／ YES→S3へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>S2a</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>余裕（MER−分岐）&gt; 0 か？</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>NO→減額 ／ YES→S2bへ（黒字なので単純な減額はしない）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>S2b</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>その予算を「目標MER超え×消化率95%以上」の商品に回した方が利益が大きいか？</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>YES→停止して転用（機会費用で負けている） ／ NO→維持し、CR・LP・価格で手当て</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>直近2日の消化率 ≥ 95% か？</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>NO→枠が余っている。増額しても消化できない→据置 ／ YES→S4へ（枠で止まっている）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>増分MERを測定済みか？</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>未測定→+25%増額（機会を取りにいくと同時に測定可能にする） ／ 測定済→S5へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>増分MER と しきい値の比較</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>≥目標MER→+20〜30%増額 ／ 分岐≤増分&lt;目標→据置（利益は増えるが利益率が下がる） ／ &lt;分岐→元の予算に戻す</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>【CRフロー】予算フローとは独立に判定する</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>悪化の先行指標が出ているか？</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>頻度&gt;2.5 ／ CTR2週連続低下 ／ 余裕3日連続縮小 ／ 7日利益2週連続減。NO→健全な商品はCRも触らない</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>新素材はあるか？</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>YES→既存広告セットに追加し判定日を+7日リセット ／ NO→複製リセット・価格・オーディエンス替えで代替</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>【増分MERの算出】Δ売上(曜日補正後) ÷ Δ広告費</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>|Δ広告費| ≥ 3,000円/日 か？</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>未満は分母が小さく値が発散するため測定しない</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>予算を意図的に変えたか？</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>変えていない場合、消化の増減はMetaのペーシング。成績が悪い日に自動で絞る逆因果を含むため実験にならない</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>P1・P2とも予算変更日をまたいでいないか？</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>またぐと変更前後が混ざり測定にならない</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>曜日構成を補正したか？</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>P1とP2の曜日指数の平均比で後期間の売上を補正する。補正しないと結論が反転する</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>■ 本日の全商品トレース（どの分岐を通ってその結論になったか）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>商品</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>日販</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>7日利益</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>MER</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>目標MER</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>分岐</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>余裕</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>消化率</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>増分MER</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>判定日</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>現予算</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>提案予算</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>結論</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>通った分岐</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>4WAY 取り付けOK 小型瞬間冷却ハンディファン</t>
+        </is>
+      </c>
+      <c r="B28" s="28" t="n">
+        <v>64.42857142857143</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>895756</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="H28" s="29" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>95000</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>95000</v>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/28）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>形状記憶日傘</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="n">
+        <v>41.28571428571428</v>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>641129</v>
+      </c>
+      <c r="D29" s="16" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="E29" s="16" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="F29" s="16" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="G29" s="16" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="H29" s="31" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>なし(健全)</t>
+        </is>
+      </c>
+      <c r="K29" s="14" t="n">
+        <v>60000</v>
+      </c>
+      <c r="L29" s="14" t="n">
+        <v>60000</v>
+      </c>
+      <c r="M29" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 なし(健全)）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>害虫ブロッカー</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="n">
+        <v>50.14285714285715</v>
+      </c>
+      <c r="C30" s="34" t="n">
+        <v>593344</v>
+      </c>
+      <c r="D30" s="35" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E30" s="35" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F30" s="35" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="G30" s="35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H30" s="36" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="I30" s="32" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J30" s="32" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="K30" s="34" t="n">
+        <v>73000</v>
+      </c>
+      <c r="L30" s="34" t="n">
+        <v>91250</v>
+      </c>
+      <c r="M30" s="32" t="inlineStr">
+        <is>
+          <t>🚀 +25%増額（測定も兼ねる）</t>
+        </is>
+      </c>
+      <c r="N30" s="37" t="inlineStr">
+        <is>
+          <t>S-1:本日が判定日 → S0:日販50.1個 → S1:7日利益+593,344円→黒字 → S2:MER 2.78 ≥ 目標 2.31→効率OK → S3:消化率102%≥95%→枠で止まっている → S4:増分MER未測定→+25%で測定可能にする</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>ナノガラス脱毛パッド</t>
+        </is>
+      </c>
+      <c r="B31" s="33" t="n">
+        <v>32.28571428571428</v>
+      </c>
+      <c r="C31" s="34" t="n">
+        <v>352962</v>
+      </c>
+      <c r="D31" s="35" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F31" s="35" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G31" s="35" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="H31" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="35" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="J31" s="32" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="K31" s="34" t="n">
+        <v>60000</v>
+      </c>
+      <c r="L31" s="34" t="n">
+        <v>75000</v>
+      </c>
+      <c r="M31" s="32" t="inlineStr">
+        <is>
+          <t>🚀 +20〜30%増額</t>
+        </is>
+      </c>
+      <c r="N31" s="37" t="inlineStr">
+        <is>
+          <t>S-1:本日が判定日 → S0:日販32.3個 → S1:7日利益+352,962円→黒字 → S2:MER 2.39 ≥ 目標 2.17→効率OK → S3:消化率100%≥95%→枠で止まっている → S4:増分MER測定済 +3.05 → S5:3.05 ≥ 目標2.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>卓上冷感クーラー</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="n">
+        <v>18.42857142857143</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>318520</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="E32" s="11" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G32" s="11" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="I32" s="11" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>7/27</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="n">
+        <v>38000</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>38000</v>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/27）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>完全遮光・形状記憶・晴雨兼用・UV日傘</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="n">
+        <v>19.85714285714286</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>260177</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E33" s="16" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G33" s="16" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H33" s="31" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I33" s="16" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="K33" s="14" t="n">
+        <v>41000</v>
+      </c>
+      <c r="L33" s="14" t="n">
+        <v>41000</v>
+      </c>
+      <c r="M33" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N33" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/28）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>接触冷感UVパーカー</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="n">
+        <v>22.14285714285714</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>178079</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G34" s="11" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="H34" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>34000</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>34000</v>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/28）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>5WAY腰掛けファン</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="n">
+        <v>11.28571428571429</v>
+      </c>
+      <c r="C35" s="14" t="n">
+        <v>170979</v>
+      </c>
+      <c r="D35" s="16" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="E35" s="16" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="H35" s="31" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="I35" s="16" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="K35" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="L35" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="M35" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N35" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/28）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>3WAYサーキュレーター扇風機</t>
+        </is>
+      </c>
+      <c r="B36" s="28" t="n">
+        <v>7.285714285714286</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>76293</v>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="F36" s="11" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="H36" s="29" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>なし(健全)</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 なし(健全)）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>偏光・調光サングラス</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="n">
+        <v>9.571428571428571</v>
+      </c>
+      <c r="C37" s="14" t="n">
+        <v>52977</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="E37" s="16" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F37" s="16" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G37" s="16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H37" s="31" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>7/29</t>
+        </is>
+      </c>
+      <c r="K37" s="14" t="n">
+        <v>22000</v>
+      </c>
+      <c r="L37" s="14" t="n">
+        <v>22000</v>
+      </c>
+      <c r="M37" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/29）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ムダ毛シェーバー</t>
+        </is>
+      </c>
+      <c r="B38" s="28" t="n">
+        <v>5.428571428571429</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>30190</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F38" s="11" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="G38" s="11" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H38" s="29" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>7/27</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="n">
+        <v>13000</v>
+      </c>
+      <c r="L38" s="6" t="n">
+        <v>13000</v>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/27）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>接触冷感UVアームカバー</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="n">
+        <v>8.142857142857142</v>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>63366</v>
+      </c>
+      <c r="D39" s="16" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="E39" s="16" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G39" s="16" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H39" s="31" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J39" s="13" t="inlineStr">
+        <is>
+          <t>7/29</t>
+        </is>
+      </c>
+      <c r="K39" s="14" t="n">
+        <v>17000</v>
+      </c>
+      <c r="L39" s="14" t="n">
+        <v>17000</v>
+      </c>
+      <c r="M39" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N39" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/29）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>瞬間冷感ポンチョ</t>
+        </is>
+      </c>
+      <c r="B40" s="28" t="n">
+        <v>7.428571428571429</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>65132</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="E40" s="11" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F40" s="11" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G40" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H40" s="29" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>8/1</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="n">
+        <v>13000</v>
+      </c>
+      <c r="L40" s="6" t="n">
+        <v>13000</v>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N40" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 8/1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>健康サンダル</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="n">
+        <v>4.857142857142857</v>
+      </c>
+      <c r="C41" s="14" t="n">
+        <v>48865</v>
+      </c>
+      <c r="D41" s="16" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="E41" s="16" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="G41" s="16" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="H41" s="31" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>なし(健全)</t>
+        </is>
+      </c>
+      <c r="K41" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="L41" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="M41" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N41" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 なし(健全)）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>携帯電動シェーバー</t>
+        </is>
+      </c>
+      <c r="B42" s="28" t="n">
+        <v>4.428571428571429</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>28532</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="F42" s="11" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="H42" s="29" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>8/1</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="n">
+        <v>11000</v>
+      </c>
+      <c r="L42" s="6" t="n">
+        <v>11000</v>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N42" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 8/1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>UV歯ブラシ除菌器</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="n">
+        <v>2.142857142857143</v>
+      </c>
+      <c r="C43" s="14" t="n">
+        <v>5614</v>
+      </c>
+      <c r="D43" s="16" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="E43" s="16" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="F43" s="16" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G43" s="16" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H43" s="31" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>7/30</t>
+        </is>
+      </c>
+      <c r="K43" s="14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="L43" s="14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M43" s="13" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N43" s="17" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/30）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>壁掛けディスペンサー</t>
+        </is>
+      </c>
+      <c r="B44" s="28" t="n">
+        <v>2.142857142857143</v>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>-22107</v>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="F44" s="11" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G44" s="11" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="H44" s="29" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>8/1</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L44" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N44" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 8/1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>湯上がりガーゼワンピース</t>
+        </is>
+      </c>
+      <c r="B45" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" s="34" t="n">
+        <v>4633</v>
+      </c>
+      <c r="D45" s="35" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="E45" s="35" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F45" s="35" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G45" s="35" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H45" s="36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I45" s="32" t="inlineStr">
+        <is>
+          <t>未測定</t>
+        </is>
+      </c>
+      <c r="J45" s="32" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="K45" s="34" t="n">
+        <v>6500</v>
+      </c>
+      <c r="L45" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="32" t="inlineStr">
+        <is>
+          <t>🔄 停止して予算を転用</t>
+        </is>
+      </c>
+      <c r="N45" s="37" t="inlineStr">
+        <is>
+          <t>S-1:本日が判定日 → S0:日販2.0個（&lt;10 利益率は参考値扱い） → S1:7日利益+4,633円→黒字 → S2:MER 1.66 &lt; 目標 3.24 → S2a:余裕+0.14&gt;0 → S2b:転用時+4,112円/日 &gt; 現状+662円/日→転用</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>バランスケアスリッパ</t>
+        </is>
+      </c>
+      <c r="B46" s="28" t="n">
+        <v>2.285714285714286</v>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>6484</v>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="E46" s="11" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="F46" s="11" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G46" s="11" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H46" s="29" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="I46" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>7/29</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L46" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>👀 据置（監視のみ）</t>
+        </is>
+      </c>
+      <c r="N46" s="12" t="inlineStr">
+        <is>
+          <t>S-1:本日は判定日ではない（次回 7/29）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>